<commit_message>
feat(oncohealth): eligibility-flat SVG with Silver column + sprint 26.04.28 ADO update
- gen-eligibility-flat-v2.js: synced COLUMNS against Miro export (103 cols), added Silver/Databricks column (OK/WARN/EXCL/NEW badges), corrected field mappings (is_medicare_advantage_risk_patient, is_erisa, is_fehb_plan, dual_eligibility_indicator)
- eligibility-flat-miro-v2.svg: regenerated 1060x4116px diagram
- knowledge.json v1.34.0: added ado_sprint_26_04_28 block (#187416 Active, #188109 new Investigation task), updated critical decisions entry, noted Nick Foreyt schema complete declaration 2026-04-21
- ADO, Confluence, Teams, gcal, SharePoint, Miro output files refreshed (2026-04-20/21 capture)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/clients/oncohealth/output/downloads/newUM_RAID.xlsx
+++ b/clients/oncohealth/output/downloads/newUM_RAID.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29912"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30006"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://oncologyanalyticsinc.sharepoint.com/sites/OncoHealth_NewFire/Shared Documents/Project Management/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="821" documentId="11_EC940C6664D167FA5349EE04A96E97124A5BFA29" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1D6F9870-1564-4AE4-B1C5-5CD46984B31A}"/>
+  <xr:revisionPtr revIDLastSave="1022" documentId="11_EC940C6664D167FA5349EE04A96E97124A5BFA29" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{02F8758D-9A45-456A-AEB6-3F15E4FF760F}"/>
   <bookViews>
-    <workbookView xWindow="2040" yWindow="390" windowWidth="26550" windowHeight="14700" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2040" yWindow="390" windowWidth="26550" windowHeight="14700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RAID Template" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="Definitions" sheetId="2" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'RAID Template'!$A$1:$Z$103</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'RAID Template'!$A$1:$Z$1</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -80,7 +80,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="221">
   <si>
     <t>Item</t>
   </si>
@@ -200,13 +200,10 @@
 not enough service code gets exercised before cutover</t>
   </si>
   <si>
-    <t>Open</t>
-  </si>
-  <si>
     <t>Analysis meeting first</t>
   </si>
   <si>
-    <t>Break apart. Mtg request to update/define risk now with design docs drafted. Tgt w/o 3/2</t>
+    <t>4/14: To be raised and reviewed with Erik/Team to determine if ARB &amp; Design Docs address this Risk. Tgt next steps by 4/17. Break apart. Mtg request to update/define risk now with design docs drafted. Tgt w/o 3/2</t>
   </si>
   <si>
     <t>Decision</t>
@@ -334,6 +331,9 @@
     <t>Any Rules Engine will need to make some assumptions about what kinds of rules can be defined and how they execute. The attached doc contains our current knowledge of how this relates to architectural and business needs.</t>
   </si>
   <si>
+    <t>Open</t>
+  </si>
+  <si>
     <t>Rules Engine Edge Cases.docx</t>
   </si>
   <si>
@@ -343,7 +343,7 @@
     <t>Develop fully functional reference</t>
   </si>
   <si>
-    <t xml:space="preserve">Action with Neal. 3/11: Confirmed with Neal, Solid progress so far, the team should have access to begin integration by 3/31; the timestamps generated may not be totally accurate but the results will start flowing through.  Related to #7 Decision, keep one.
+    <t xml:space="preserve">4/7: Per feedback from Donato, knowledge transfer happened and Services team knows what to do. Closing this risk. Action with Neal. 3/11: Confirmed with Neal, Solid progress so far, the team should have access to begin integration by 3/31; the timestamps generated may not be totally accurate but the results will start flowing through.  Related to #7 Decision, keep one.
 2/27: Keep. Fully functional reference due by 3/31. Donato/Neal/Matt have been in contact. An implementation call is to be scheduled. </t>
   </si>
   <si>
@@ -374,7 +374,7 @@
     <t>Marc Gale</t>
   </si>
   <si>
-    <t>3/6: draft doc uploaded to SP for review. 2/27: Task to schedule call (Donato) for next week so group can align on scenarios, risks and sequencing. 2/20: discussed in project team mtg. Next step is to identify first client (tgt end of Feb). Then team will need to regroup to determine approach. Will remain In Progress; update can be made after 1st client identified.</t>
+    <t>4/2: Update - (Alison) proposal discussed on 3/31. Need additional week as team was focused on NCAQ audit. Will discuss on 4/7. 3/6: draft doc uploaded to SP for review. 2/27: Task to schedule call (Donato) for next week so group can align on scenarios, risks and sequencing. 2/20: discussed in project team mtg. Next step is to identify first client (tgt end of Feb). Then team will need to regroup to determine approach. Will remain In Progress; update can be made after 1st client identified.</t>
   </si>
   <si>
     <t>Newfire data team wasn't aware of the shortcomings of OH's process of masking PHI. This had been noted several times in earlier meetings</t>
@@ -418,7 +418,7 @@
     <t>Requirements  &amp; Change Request decision</t>
   </si>
   <si>
-    <t>3/6: Venky noted team is about 2 weeks away from fully defining all the data elements that we are going to get.  Evaluate when ready, determine if a Risk or a CR that needs to be created. Notes: expose public endpoints for our APIs for case entry and (2) we have to make sure there's the idea of provided-but-not-validated data so the CSR can approve the new case and validate the data provided</t>
+    <t>4/13: Per Venky, put off conversation until we have R1 released.  4/7: Target follow up week of 4/13. 3/25: per ESC, revisit in April. 3/6: Venky noted team is about 2 weeks away from fully defining all the data elements that we are going to get.  Evaluate when ready, determine if a Risk or a CR that needs to be created. Notes: expose public endpoints for our APIs for case entry and (2) we have to make sure there's the idea of provided-but-not-validated data so the CSR can approve the new case and validate the data provided</t>
   </si>
   <si>
     <t>BAs need to create 60 PRDs for R2 in preparation for the PI planning (2 per day)</t>
@@ -427,7 +427,8 @@
     <t>Initiate Conf Specialist (BAs) role fulfillment earlier than planned. This is now in progress.</t>
   </si>
   <si>
-    <t>3/18: Staffing being reviewed; additional project resources expected to support.</t>
+    <t>4/3: 2 of 3 positions open for Tech Product Owner; starting to see candidate pipeline.
+3/18: Staffing being reviewed; additional project resources expected to support.</t>
   </si>
   <si>
     <t>Team needs to deliver 60 PRDs for R2 (2 per day). Taking into account results of 1st PI planning (8 for PI), this looks like risk</t>
@@ -451,10 +452,11 @@
     <t>Donato Buccella</t>
   </si>
   <si>
-    <t>waiting on exec sign-off</t>
-  </si>
-  <si>
-    <t>https://oncologyanalyticsinc-my.sharepoint.com/:w:/g/personal/jhall_oncologyanalytics_com/IQD0DSuZtNiXSa6uU3iYJNI7AdkBslIlyHhXlHPWDLdb_Pw?e=60ofzr</t>
+    <t>waiting on exec sign-off; 
+https://oncologyanalyticsinc-my.sharepoint.com/:w:/g/personal/jhall_oncologyanalytics_com/IQD0DSuZtNiXSa6uU3iYJNI7AdkBslIlyHhXlHPWDLdb_Pw?e=60ofzr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Per Salin, 3/23: We should be covered from both Security and DevOps perspectives. Security has no concerns about which service we build, as long as it's hosted in OH approved Azure region. </t>
   </si>
   <si>
     <t>Geisinger selected as first client for NewUM</t>
@@ -463,6 +465,24 @@
     <t>Sandy shared presentation at 2/27 meeting; team moving forward with decision.</t>
   </si>
   <si>
+    <t>Issue</t>
+  </si>
+  <si>
+    <t>Product Team needs to review PRDs and provide input for #28. Limited resources</t>
+  </si>
+  <si>
+    <t>Raising at 3/13 meeting</t>
+  </si>
+  <si>
+    <t>Monitor</t>
+  </si>
+  <si>
+    <t>Ann Dye</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3/12- Will discuss in weekly team call. </t>
+  </si>
+  <si>
     <t>The test automation architecture and technology stack for both API and UI automation, shared on 3/11, does not clearly demonstrate alignment with OncoHealth’s expectations for a simple, maintainable, and supportable framework. OncoHealth is seeking a streamlined approach for API and UI automation that aligns with proven patterns and supports long‑term sustainability, scalability, and ease of adoption across teams.</t>
   </si>
   <si>
@@ -475,19 +495,95 @@
     <t>Configuration rework will potentially push the schedule out.</t>
   </si>
   <si>
-    <t>Ann Dye</t>
-  </si>
-  <si>
-    <t>Issue</t>
-  </si>
-  <si>
-    <t>Product Team needs to review PRDs and provide input for #28. Limited resources</t>
-  </si>
-  <si>
-    <t>Raising at 3/13 meeting</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3/12- Will discuss in weekly team call. </t>
+    <t xml:space="preserve">Risk </t>
+  </si>
+  <si>
+    <t>Completing the Happy Path Prototype Review by 4/3 is a challenge and will put other UX/UI work on hold.</t>
+  </si>
+  <si>
+    <t>Parallel work continues</t>
+  </si>
+  <si>
+    <t>4/1: Will review progress on 4/2
+4/17: Parallel work has continued and insights/feedback gained from the prototyping happy path effort have been a net positive for the design process.</t>
+  </si>
+  <si>
+    <t>We will have admin pages and funcitonality in NewUM, and where needed we can work with OH to extend any changes needed in Admin app (used for external service management and config)</t>
+  </si>
+  <si>
+    <t>Raised in 3/23 check-in call. In about 4 weeks we should be evaluating the detailed configuration design</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Using a write-only table to store/version Eligibility records may cause performance problems when performing an eligibility search on case intake. </t>
+  </si>
+  <si>
+    <t>Michal Mucha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Populate the new Eligibility table with synthetic data based on the conditional distributions of key IDs and dates. Use this synthetic data to do performance tests, and adjust partitioning and indexing as needed. If no viable partitioning/indexing solution exists (which is very unlikely), consider creating a separate table for current eligibility records. </t>
+  </si>
+  <si>
+    <t>Service Integration Design: Document Management Service</t>
+  </si>
+  <si>
+    <t>Matthew Emerson</t>
+  </si>
+  <si>
+    <t>https://oncologyanalyticsinc.sharepoint.com/:w:/r/sites/OncoHealth_NewFire/_layouts/15/Doc.aspx?sourcedoc=%7B8B891A0D-0949-4088-A6CD-8ED34088A9A7%7D&amp;file=NewUM%25u00a0Services%20Integration%20Design.docx&amp;action=default&amp;mobileredirect=true</t>
+  </si>
+  <si>
+    <t>4/6/26 decision Option C, see document</t>
+  </si>
+  <si>
+    <t>Service Integration Design:Drugs API</t>
+  </si>
+  <si>
+    <t>Service Integration Design:Eligibility Service</t>
+  </si>
+  <si>
+    <t>4/6/26 decision Option B, see document</t>
+  </si>
+  <si>
+    <t>Service Integration Design:Fax Service</t>
+  </si>
+  <si>
+    <t>Service Integration Design: Job Monitor</t>
+  </si>
+  <si>
+    <t>4/8/26 decision Option C, see document</t>
+  </si>
+  <si>
+    <t>Service Integration Design: Kaleidoscope</t>
+  </si>
+  <si>
+    <t>4/8/26 decision Option B, see document</t>
+  </si>
+  <si>
+    <t>Service Integration Design: Letters V2</t>
+  </si>
+  <si>
+    <t>4/8/26 decision Option A, see document</t>
+  </si>
+  <si>
+    <t>Service Integration Design:Okta</t>
+  </si>
+  <si>
+    <t>Service Integration Design: TAT API &amp; Chronos</t>
+  </si>
+  <si>
+    <t>Service Integration Design: Twilio</t>
+  </si>
+  <si>
+    <t>Unclear understanding of potential changes to Drugs API</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Team to meet to discuss further for planning &amp; alignment. Jason raised during project working team call. </t>
+  </si>
+  <si>
+    <t>Fax intake technical &amp; process approach not yet understood</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Team to meet to discuss further for planning &amp; alignment.Eirk/Jason raised during project working team call. </t>
   </si>
   <si>
     <t>Item/ Deliverable</t>
@@ -853,7 +949,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -881,16 +977,12 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1192,7 +1284,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr>
+  <sheetPr filterMode="1">
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:Z103"/>
@@ -1268,7 +1360,7 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="2" spans="1:26" ht="48">
+    <row r="2" spans="1:26" ht="48" hidden="1">
       <c r="A2" s="10">
         <v>1</v>
       </c>
@@ -1313,7 +1405,7 @@
         <v>46080</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="84">
+    <row r="3" spans="1:26" ht="84" hidden="1">
       <c r="A3" s="11">
         <v>2</v>
       </c>
@@ -1358,7 +1450,7 @@
         <v>46087</v>
       </c>
     </row>
-    <row r="4" spans="1:26" ht="96">
+    <row r="4" spans="1:26" ht="72">
       <c r="A4" s="11">
         <v>3</v>
       </c>
@@ -1378,7 +1470,7 @@
         <v>2</v>
       </c>
       <c r="G4" s="14">
-        <f t="shared" si="0"/>
+        <f>E4*F4</f>
         <v>8</v>
       </c>
       <c r="H4" s="11" t="s">
@@ -1401,7 +1493,7 @@
       </c>
       <c r="N4" s="13"/>
     </row>
-    <row r="5" spans="1:26" ht="72">
+    <row r="5" spans="1:26" ht="60">
       <c r="A5" s="11">
         <v>4</v>
       </c>
@@ -1421,7 +1513,7 @@
         <v>4</v>
       </c>
       <c r="G5" s="14">
-        <f t="shared" si="0"/>
+        <f>E5*F5</f>
         <v>16</v>
       </c>
       <c r="H5" s="11" t="s">
@@ -1444,7 +1536,7 @@
       </c>
       <c r="N5" s="13"/>
     </row>
-    <row r="6" spans="1:26" ht="36">
+    <row r="6" spans="1:26" ht="72">
       <c r="A6" s="11">
         <v>5</v>
       </c>
@@ -1464,16 +1556,16 @@
         <v>3</v>
       </c>
       <c r="G6" s="14">
-        <f t="shared" si="0"/>
+        <f>E6*F6</f>
         <v>12</v>
       </c>
       <c r="H6" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="I6" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="I6" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="J6" s="11" t="s">
+      <c r="J6" s="2" t="s">
         <v>19</v>
       </c>
       <c r="K6" s="15">
@@ -1483,19 +1575,19 @@
         <v>16</v>
       </c>
       <c r="M6" s="12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="N6" s="13"/>
     </row>
-    <row r="7" spans="1:26" ht="96">
+    <row r="7" spans="1:26" ht="96" hidden="1">
       <c r="A7" s="10">
         <v>6</v>
       </c>
       <c r="B7" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="C7" s="12" t="s">
         <v>38</v>
-      </c>
-      <c r="C7" s="12" t="s">
-        <v>39</v>
       </c>
       <c r="D7" s="13" t="s">
         <v>26</v>
@@ -1503,7 +1595,7 @@
       <c r="E7" s="13"/>
       <c r="F7" s="13"/>
       <c r="G7" s="14">
-        <f t="shared" si="0"/>
+        <f>E7*F7</f>
         <v>0</v>
       </c>
       <c r="H7" s="11" t="s">
@@ -1518,21 +1610,21 @@
         <v>31</v>
       </c>
       <c r="M7" s="12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="N7" s="6">
         <v>46084</v>
       </c>
     </row>
-    <row r="8" spans="1:26" ht="24">
+    <row r="8" spans="1:26" ht="24" hidden="1">
       <c r="A8" s="11">
         <v>7</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D8" s="13" t="s">
         <v>26</v>
@@ -1540,7 +1632,7 @@
       <c r="E8" s="13"/>
       <c r="F8" s="13"/>
       <c r="G8" s="14">
-        <f t="shared" si="0"/>
+        <f>E8*F8</f>
         <v>0</v>
       </c>
       <c r="H8" s="11" t="s">
@@ -1555,13 +1647,13 @@
         <v>31</v>
       </c>
       <c r="M8" s="13" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="N8" s="6">
         <v>46080</v>
       </c>
     </row>
-    <row r="9" spans="1:26" ht="25.5">
+    <row r="9" spans="1:26" ht="25.5" hidden="1">
       <c r="A9" s="11">
         <v>8</v>
       </c>
@@ -1569,7 +1661,7 @@
         <v>14</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D9" s="13" t="s">
         <v>16</v>
@@ -1581,14 +1673,14 @@
         <v>3</v>
       </c>
       <c r="G9" s="14">
-        <f t="shared" si="0"/>
+        <f>E9*F9</f>
         <v>9</v>
       </c>
       <c r="H9" s="11" t="s">
         <v>17</v>
       </c>
       <c r="I9" s="13" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="J9" s="11" t="s">
         <v>19</v>
@@ -1599,14 +1691,14 @@
       <c r="L9" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="M9" s="18" t="s">
-        <v>45</v>
+      <c r="M9" s="17" t="s">
+        <v>44</v>
       </c>
       <c r="N9" s="15">
         <v>46070</v>
       </c>
     </row>
-    <row r="10" spans="1:26" ht="72">
+    <row r="10" spans="1:26" ht="72" hidden="1">
       <c r="A10" s="11">
         <v>9</v>
       </c>
@@ -1614,10 +1706,10 @@
         <v>14</v>
       </c>
       <c r="C10" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="D10" s="13" t="s">
         <v>46</v>
-      </c>
-      <c r="D10" s="13" t="s">
-        <v>47</v>
       </c>
       <c r="E10" s="13">
         <v>4</v>
@@ -1626,14 +1718,14 @@
         <v>4</v>
       </c>
       <c r="G10" s="14">
-        <f t="shared" si="0"/>
+        <f>E10*F10</f>
         <v>16</v>
       </c>
       <c r="H10" s="11" t="s">
         <v>17</v>
       </c>
       <c r="I10" s="13" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J10" s="11" t="s">
         <v>19</v>
@@ -1645,21 +1737,21 @@
         <v>16</v>
       </c>
       <c r="M10" s="12" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="N10" s="6">
         <v>46084</v>
       </c>
     </row>
-    <row r="11" spans="1:26" ht="24">
+    <row r="11" spans="1:26" ht="24" hidden="1">
       <c r="A11" s="11">
         <v>10</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D11" s="13" t="s">
         <v>26</v>
@@ -1667,7 +1759,7 @@
       <c r="E11" s="13"/>
       <c r="F11" s="13"/>
       <c r="G11" s="14">
-        <f t="shared" si="0"/>
+        <f>E11*F11</f>
         <v>0</v>
       </c>
       <c r="H11" s="11" t="s">
@@ -1682,13 +1774,13 @@
         <v>31</v>
       </c>
       <c r="M11" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="N11" s="6">
         <v>46080</v>
       </c>
     </row>
-    <row r="12" spans="1:26" ht="84">
+    <row r="12" spans="1:26" ht="84" hidden="1">
       <c r="A12" s="10">
         <v>11</v>
       </c>
@@ -1696,7 +1788,7 @@
         <v>14</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D12" s="13" t="s">
         <v>16</v>
@@ -1708,14 +1800,14 @@
         <v>3</v>
       </c>
       <c r="G12" s="14">
-        <f t="shared" si="0"/>
+        <f>E12*F12</f>
         <v>9</v>
       </c>
       <c r="H12" s="11" t="s">
         <v>17</v>
       </c>
       <c r="I12" s="12" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J12" s="11" t="s">
         <v>19</v>
@@ -1727,13 +1819,13 @@
         <v>16</v>
       </c>
       <c r="M12" s="12" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="N12" s="6">
         <v>46080</v>
       </c>
     </row>
-    <row r="13" spans="1:26" ht="12.75">
+    <row r="13" spans="1:26" ht="12.75" hidden="1">
       <c r="A13" s="11">
         <v>12</v>
       </c>
@@ -1741,7 +1833,7 @@
         <v>14</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D13" s="13" t="s">
         <v>16</v>
@@ -1753,7 +1845,7 @@
         <v>3</v>
       </c>
       <c r="G13" s="14">
-        <f t="shared" si="0"/>
+        <f>E13*F13</f>
         <v>9</v>
       </c>
       <c r="H13" s="11" t="s">
@@ -1769,22 +1861,22 @@
       <c r="L13" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="M13" s="18" t="s">
-        <v>56</v>
+      <c r="M13" s="17" t="s">
+        <v>55</v>
       </c>
       <c r="N13" s="15">
         <v>46051</v>
       </c>
     </row>
-    <row r="14" spans="1:26" ht="12.75">
+    <row r="14" spans="1:26" ht="12.75" hidden="1">
       <c r="A14" s="11">
         <v>13</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D14" s="13" t="s">
         <v>26</v>
@@ -1792,7 +1884,7 @@
       <c r="E14" s="13"/>
       <c r="F14" s="13"/>
       <c r="G14" s="14">
-        <f t="shared" si="0"/>
+        <f>E14*F14</f>
         <v>0</v>
       </c>
       <c r="H14" s="11" t="s">
@@ -1800,7 +1892,7 @@
       </c>
       <c r="I14" s="16"/>
       <c r="J14" s="16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="K14" s="15">
         <v>46045</v>
@@ -1809,13 +1901,13 @@
         <v>31</v>
       </c>
       <c r="M14" s="13" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="N14" s="6">
         <v>46098</v>
       </c>
     </row>
-    <row r="15" spans="1:26" ht="12.75">
+    <row r="15" spans="1:26" ht="12.75" hidden="1">
       <c r="A15" s="11">
         <v>14</v>
       </c>
@@ -1823,10 +1915,10 @@
         <v>14</v>
       </c>
       <c r="C15" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="D15" s="13" t="s">
         <v>60</v>
-      </c>
-      <c r="D15" s="13" t="s">
-        <v>61</v>
       </c>
       <c r="E15" s="13">
         <v>5</v>
@@ -1835,14 +1927,14 @@
         <v>4</v>
       </c>
       <c r="G15" s="14">
-        <f t="shared" si="0"/>
+        <f>E15*F15</f>
         <v>20</v>
       </c>
       <c r="H15" s="11" t="s">
         <v>17</v>
       </c>
       <c r="I15" s="13" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="J15" s="11" t="s">
         <v>19</v>
@@ -1851,14 +1943,14 @@
         <v>46048</v>
       </c>
       <c r="L15" s="13"/>
-      <c r="M15" s="18" t="s">
-        <v>63</v>
+      <c r="M15" s="17" t="s">
+        <v>62</v>
       </c>
       <c r="N15" s="15">
         <v>46071</v>
       </c>
     </row>
-    <row r="16" spans="1:26" ht="12.75">
+    <row r="16" spans="1:26" ht="12.75" hidden="1">
       <c r="A16" s="11">
         <v>15</v>
       </c>
@@ -1866,7 +1958,7 @@
         <v>14</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D16" s="13" t="s">
         <v>16</v>
@@ -1878,14 +1970,14 @@
         <v>3</v>
       </c>
       <c r="G16" s="14">
-        <f t="shared" si="0"/>
+        <f>E16*F16</f>
         <v>15</v>
       </c>
       <c r="H16" s="11" t="s">
         <v>17</v>
       </c>
       <c r="I16" s="13" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J16" s="11" t="s">
         <v>19</v>
@@ -1896,8 +1988,8 @@
       <c r="L16" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="M16" s="18" t="s">
-        <v>66</v>
+      <c r="M16" s="17" t="s">
+        <v>65</v>
       </c>
       <c r="N16" s="15">
         <v>46063</v>
@@ -1911,7 +2003,7 @@
         <v>14</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D17" s="13" t="s">
         <v>26</v>
@@ -1923,14 +2015,14 @@
         <v>4</v>
       </c>
       <c r="G17" s="14">
-        <f t="shared" si="0"/>
+        <f>E17*F17</f>
         <v>20</v>
       </c>
       <c r="H17" s="11" t="s">
         <v>27</v>
       </c>
       <c r="I17" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="J17" s="11" t="s">
         <v>19</v>
@@ -1939,14 +2031,14 @@
         <v>46049</v>
       </c>
       <c r="L17" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="M17" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="M17" s="12" t="s">
-        <v>70</v>
-      </c>
       <c r="N17" s="13"/>
     </row>
-    <row r="18" spans="1:14" ht="25.5">
+    <row r="18" spans="1:14" ht="25.5" hidden="1">
       <c r="A18" s="11">
         <v>17</v>
       </c>
@@ -1954,10 +2046,10 @@
         <v>14</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E18" s="13">
         <v>3</v>
@@ -1966,14 +2058,14 @@
         <v>4</v>
       </c>
       <c r="G18" s="14">
-        <f t="shared" si="0"/>
+        <f>E18*F18</f>
         <v>12</v>
       </c>
       <c r="H18" s="11" t="s">
         <v>17</v>
       </c>
       <c r="I18" s="7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J18" s="11" t="s">
         <v>19</v>
@@ -1982,16 +2074,16 @@
         <v>46057</v>
       </c>
       <c r="L18" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="M18" s="18" t="s">
-        <v>73</v>
-      </c>
-      <c r="N18" s="20">
+        <v>46</v>
+      </c>
+      <c r="M18" s="17" t="s">
+        <v>72</v>
+      </c>
+      <c r="N18" s="19">
         <v>46070</v>
       </c>
     </row>
-    <row r="19" spans="1:14" ht="25.5">
+    <row r="19" spans="1:14" ht="25.5" hidden="1">
       <c r="A19" s="11">
         <v>18</v>
       </c>
@@ -1999,10 +2091,10 @@
         <v>14</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E19" s="13">
         <v>3</v>
@@ -2011,14 +2103,14 @@
         <v>3</v>
       </c>
       <c r="G19" s="14">
-        <f t="shared" si="0"/>
+        <f>E19*F19</f>
         <v>9</v>
       </c>
       <c r="H19" s="11" t="s">
         <v>17</v>
       </c>
       <c r="I19" s="7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="J19" s="11" t="s">
         <v>19</v>
@@ -2027,24 +2119,24 @@
         <v>46057</v>
       </c>
       <c r="L19" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="M19" s="18" t="s">
-        <v>76</v>
+        <v>46</v>
+      </c>
+      <c r="M19" s="17" t="s">
+        <v>75</v>
       </c>
       <c r="N19" s="15">
         <v>46070</v>
       </c>
     </row>
-    <row r="20" spans="1:14" ht="51">
+    <row r="20" spans="1:14" ht="48" hidden="1">
       <c r="A20" s="11">
         <v>19</v>
       </c>
       <c r="B20" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="C20" s="12" t="s">
         <v>77</v>
-      </c>
-      <c r="C20" s="12" t="s">
-        <v>78</v>
       </c>
       <c r="D20" s="13" t="s">
         <v>26</v>
@@ -2052,14 +2144,13 @@
       <c r="E20" s="13"/>
       <c r="F20" s="13"/>
       <c r="G20" s="14">
-        <f t="shared" si="0"/>
+        <f>E20*F20</f>
         <v>0</v>
       </c>
       <c r="H20" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="I20" s="13"/>
-      <c r="J20" s="17" t="s">
+        <v>78</v>
+      </c>
+      <c r="I20" s="16" t="s">
         <v>79</v>
       </c>
       <c r="K20" s="15">
@@ -2068,10 +2159,10 @@
       <c r="L20" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="M20" s="18"/>
+      <c r="M20" s="17"/>
       <c r="N20" s="13"/>
     </row>
-    <row r="21" spans="1:14" ht="130.5">
+    <row r="21" spans="1:14" ht="166.5" hidden="1">
       <c r="A21" s="11">
         <v>20</v>
       </c>
@@ -2091,11 +2182,11 @@
         <v>3</v>
       </c>
       <c r="G21" s="14">
-        <f t="shared" si="0"/>
+        <f>E21*F21</f>
         <v>9</v>
       </c>
       <c r="H21" s="11" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="I21" s="13" t="s">
         <v>81</v>
@@ -2109,12 +2200,14 @@
       <c r="L21" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="M21" s="19" t="s">
+      <c r="M21" s="18" t="s">
         <v>82</v>
       </c>
-      <c r="N21" s="13"/>
-    </row>
-    <row r="22" spans="1:14" ht="72">
+      <c r="N21" s="15">
+        <v>46119</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" ht="72" hidden="1">
       <c r="A22" s="11">
         <v>21</v>
       </c>
@@ -2134,7 +2227,7 @@
         <v>3</v>
       </c>
       <c r="G22" s="14">
-        <f t="shared" si="0"/>
+        <f>E22*F22</f>
         <v>12</v>
       </c>
       <c r="H22" s="11" t="s">
@@ -2150,14 +2243,14 @@
       <c r="L22" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="M22" s="19" t="s">
+      <c r="M22" s="18" t="s">
         <v>85</v>
       </c>
       <c r="N22" s="15">
         <v>46080</v>
       </c>
     </row>
-    <row r="23" spans="1:14" ht="60">
+    <row r="23" spans="1:14" ht="60" hidden="1">
       <c r="A23" s="11">
         <v>22</v>
       </c>
@@ -2168,7 +2261,7 @@
         <v>86</v>
       </c>
       <c r="D23" s="12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E23" s="13">
         <v>3</v>
@@ -2177,7 +2270,7 @@
         <v>4</v>
       </c>
       <c r="G23" s="14">
-        <f t="shared" si="0"/>
+        <f>E23*F23</f>
         <v>12</v>
       </c>
       <c r="H23" s="11" t="s">
@@ -2193,16 +2286,16 @@
         <v>46070</v>
       </c>
       <c r="L23" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="M23" s="19" t="s">
+        <v>46</v>
+      </c>
+      <c r="M23" s="18" t="s">
         <v>88</v>
       </c>
       <c r="N23" s="15">
         <v>46076</v>
       </c>
     </row>
-    <row r="24" spans="1:14" ht="118.5">
+    <row r="24" spans="1:14" ht="154.5">
       <c r="A24" s="10">
         <v>23</v>
       </c>
@@ -2222,7 +2315,7 @@
         <v>3</v>
       </c>
       <c r="G24" s="14">
-        <f t="shared" si="0"/>
+        <f>E24*F24</f>
         <v>6</v>
       </c>
       <c r="H24" s="11" t="s">
@@ -2240,12 +2333,12 @@
       <c r="L24" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="M24" s="19" t="s">
+      <c r="M24" s="18" t="s">
         <v>92</v>
       </c>
       <c r="N24" s="13"/>
     </row>
-    <row r="25" spans="1:14" ht="60">
+    <row r="25" spans="1:14" ht="48">
       <c r="A25" s="11">
         <v>24</v>
       </c>
@@ -2265,7 +2358,7 @@
         <v>3</v>
       </c>
       <c r="G25" s="14">
-        <f t="shared" si="0"/>
+        <f>E25*F25</f>
         <v>6</v>
       </c>
       <c r="H25" s="11" t="s">
@@ -2283,12 +2376,12 @@
       <c r="L25" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="M25" s="19" t="s">
+      <c r="M25" s="18" t="s">
         <v>95</v>
       </c>
       <c r="N25" s="13"/>
     </row>
-    <row r="26" spans="1:14" ht="38.25">
+    <row r="26" spans="1:14" ht="38.25" hidden="1">
       <c r="A26" s="11">
         <v>25</v>
       </c>
@@ -2304,7 +2397,7 @@
       <c r="E26" s="13"/>
       <c r="F26" s="13"/>
       <c r="G26" s="14">
-        <f t="shared" si="0"/>
+        <f>E26*F26</f>
         <v>0</v>
       </c>
       <c r="H26" s="11" t="s">
@@ -2322,12 +2415,12 @@
       <c r="L26" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="M26" s="18"/>
+      <c r="M26" s="17"/>
       <c r="N26" s="15">
         <v>46070</v>
       </c>
     </row>
-    <row r="27" spans="1:14" ht="107.25">
+    <row r="27" spans="1:14" ht="107.25" hidden="1">
       <c r="A27" s="11">
         <v>26</v>
       </c>
@@ -2338,7 +2431,7 @@
         <v>99</v>
       </c>
       <c r="D27" s="13" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E27" s="13">
         <v>2</v>
@@ -2347,7 +2440,7 @@
         <v>3</v>
       </c>
       <c r="G27" s="14">
-        <f t="shared" si="0"/>
+        <f>E27*F27</f>
         <v>6</v>
       </c>
       <c r="H27" s="11" t="s">
@@ -2365,14 +2458,14 @@
       <c r="L27" s="13" t="s">
         <v>101</v>
       </c>
-      <c r="M27" s="19" t="s">
+      <c r="M27" s="18" t="s">
         <v>102</v>
       </c>
       <c r="N27" s="15">
         <v>46080</v>
       </c>
     </row>
-    <row r="28" spans="1:14" ht="154.5">
+    <row r="28" spans="1:14" ht="166.5" hidden="1">
       <c r="A28" s="11">
         <v>27</v>
       </c>
@@ -2392,7 +2485,7 @@
         <v>1</v>
       </c>
       <c r="G28" s="14">
-        <f t="shared" si="0"/>
+        <f>E28*F28</f>
         <v>4</v>
       </c>
       <c r="H28" s="11" t="s">
@@ -2408,12 +2501,12 @@
       <c r="L28" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="M28" s="19" t="s">
+      <c r="M28" s="18" t="s">
         <v>106</v>
       </c>
       <c r="N28" s="13"/>
     </row>
-    <row r="29" spans="1:14" ht="24">
+    <row r="29" spans="1:14" ht="48">
       <c r="A29" s="11">
         <v>28</v>
       </c>
@@ -2433,7 +2526,7 @@
         <v>4</v>
       </c>
       <c r="G29" s="14">
-        <f t="shared" si="0"/>
+        <f>E29*F29</f>
         <v>20</v>
       </c>
       <c r="H29" s="11" t="s">
@@ -2449,14 +2542,14 @@
         <v>46080</v>
       </c>
       <c r="L29" s="13" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="M29" s="18" t="s">
         <v>109</v>
       </c>
       <c r="N29" s="13"/>
     </row>
-    <row r="30" spans="1:14" ht="36.75" customHeight="1">
+    <row r="30" spans="1:14" ht="36.75" hidden="1" customHeight="1">
       <c r="A30" s="11">
         <v>29</v>
       </c>
@@ -2472,11 +2565,11 @@
       <c r="E30" s="13"/>
       <c r="F30" s="13"/>
       <c r="G30" s="14">
-        <f t="shared" si="0"/>
+        <f>E30*F30</f>
         <v>0</v>
       </c>
       <c r="H30" s="11" t="s">
-        <v>35</v>
+        <v>78</v>
       </c>
       <c r="I30" s="13" t="s">
         <v>111</v>
@@ -2486,17 +2579,17 @@
         <v>46080</v>
       </c>
       <c r="L30" s="13" t="s">
-        <v>61</v>
-      </c>
-      <c r="M30" s="18"/>
+        <v>60</v>
+      </c>
+      <c r="M30" s="17"/>
       <c r="N30" s="13"/>
     </row>
-    <row r="31" spans="1:14" ht="36">
+    <row r="31" spans="1:14" ht="36" hidden="1">
       <c r="A31" s="10">
         <v>30</v>
       </c>
       <c r="B31" s="11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C31" s="12" t="s">
         <v>112</v>
@@ -2505,7 +2598,7 @@
       <c r="E31" s="13"/>
       <c r="F31" s="13"/>
       <c r="G31" s="14">
-        <f t="shared" si="0"/>
+        <f>E31*F31</f>
         <v>0</v>
       </c>
       <c r="H31" s="11" t="s">
@@ -2519,19 +2612,19 @@
       <c r="L31" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="M31" s="18" t="s">
+      <c r="M31" s="17" t="s">
         <v>113</v>
       </c>
       <c r="N31" s="15">
         <v>46080</v>
       </c>
     </row>
-    <row r="32" spans="1:14" ht="12.75">
+    <row r="32" spans="1:14" ht="12.75" hidden="1">
       <c r="A32" s="11">
         <v>31</v>
       </c>
       <c r="B32" s="11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C32" s="12" t="s">
         <v>114</v>
@@ -2542,7 +2635,7 @@
       <c r="E32" s="13"/>
       <c r="F32" s="13"/>
       <c r="G32" s="14">
-        <f t="shared" si="0"/>
+        <f>E32*F32</f>
         <v>0</v>
       </c>
       <c r="H32" s="11" t="s">
@@ -2556,17 +2649,17 @@
       <c r="L32" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="M32" s="23"/>
-      <c r="N32" s="20">
+      <c r="M32" s="21"/>
+      <c r="N32" s="19">
         <v>46084</v>
       </c>
     </row>
-    <row r="33" spans="1:14" ht="60">
+    <row r="33" spans="1:14" ht="72" hidden="1">
       <c r="A33" s="11">
         <v>32</v>
       </c>
       <c r="B33" s="11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C33" s="12" t="s">
         <v>115</v>
@@ -2578,29 +2671,31 @@
       <c r="F33" s="13"/>
       <c r="G33" s="14"/>
       <c r="H33" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="I33" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="I33" s="12" t="s">
         <v>117</v>
       </c>
       <c r="J33" s="11"/>
       <c r="K33" s="15">
         <v>46084</v>
       </c>
-      <c r="L33" s="18" t="s">
+      <c r="L33" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="M33" s="22" t="s">
+      <c r="M33" s="17" t="s">
         <v>118</v>
       </c>
-      <c r="N33" s="13"/>
-    </row>
-    <row r="34" spans="1:14" ht="12.75">
+      <c r="N33" s="15">
+        <v>46104</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14" ht="12.75" hidden="1">
       <c r="A34" s="11">
         <v>33</v>
       </c>
       <c r="B34" s="11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C34" s="12" t="s">
         <v>119</v>
@@ -2609,7 +2704,7 @@
       <c r="E34" s="13"/>
       <c r="F34" s="13"/>
       <c r="G34" s="14">
-        <f t="shared" si="0"/>
+        <f>E34*F34</f>
         <v>0</v>
       </c>
       <c r="H34" s="11"/>
@@ -2621,416 +2716,698 @@
       <c r="L34" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="M34" s="21" t="s">
+      <c r="M34" s="20" t="s">
         <v>120</v>
       </c>
-      <c r="N34" s="24">
+      <c r="N34" s="22">
         <v>46085</v>
       </c>
     </row>
-    <row r="35" spans="1:14" ht="98.25" customHeight="1">
+    <row r="35" spans="1:14" ht="98.25" hidden="1" customHeight="1">
       <c r="A35" s="11">
+        <v>38</v>
+      </c>
+      <c r="B35" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="C35" s="18" t="s">
+        <v>122</v>
+      </c>
+      <c r="D35" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="E35" s="13">
+        <v>5</v>
+      </c>
+      <c r="F35" s="13">
+        <v>5</v>
+      </c>
+      <c r="G35" s="13">
+        <v>25</v>
+      </c>
+      <c r="H35" s="13" t="s">
+        <v>78</v>
+      </c>
+      <c r="I35" s="13" t="s">
+        <v>123</v>
+      </c>
+      <c r="J35" s="13" t="s">
+        <v>124</v>
+      </c>
+      <c r="K35" s="15">
+        <v>46093</v>
+      </c>
+      <c r="L35" s="13" t="s">
+        <v>125</v>
+      </c>
+      <c r="M35" s="17" t="s">
+        <v>126</v>
+      </c>
+      <c r="N35" s="13"/>
+    </row>
+    <row r="36" spans="1:14" ht="85.5" hidden="1">
+      <c r="A36" s="11">
         <v>34</v>
-      </c>
-      <c r="B35" s="11"/>
-      <c r="C35" s="19" t="s">
-        <v>121</v>
-      </c>
-      <c r="D35" s="13"/>
-      <c r="E35" s="13"/>
-      <c r="F35" s="13"/>
-      <c r="G35" s="14">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H35" s="11" t="s">
-        <v>104</v>
-      </c>
-      <c r="I35" s="13"/>
-      <c r="J35" s="11"/>
-      <c r="K35" s="15">
-        <v>46094</v>
-      </c>
-      <c r="L35" s="13" t="s">
-        <v>122</v>
-      </c>
-      <c r="M35" s="18" t="s">
-        <v>123</v>
-      </c>
-      <c r="N35" s="13"/>
-    </row>
-    <row r="36" spans="1:14" ht="12.75">
-      <c r="A36" s="11">
-        <v>35</v>
       </c>
       <c r="B36" s="11"/>
       <c r="C36" s="12" t="s">
-        <v>124</v>
-      </c>
-      <c r="D36" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="E36" s="13">
-        <v>4</v>
-      </c>
-      <c r="F36" s="13">
-        <v>5</v>
-      </c>
+        <v>127</v>
+      </c>
+      <c r="D36" s="13"/>
+      <c r="E36" s="13"/>
+      <c r="F36" s="13"/>
       <c r="G36" s="14">
-        <f t="shared" si="0"/>
-        <v>20</v>
+        <f>E36*F36</f>
+        <v>0</v>
       </c>
       <c r="H36" s="11" t="s">
-        <v>27</v>
+        <v>104</v>
       </c>
       <c r="I36" s="13"/>
       <c r="J36" s="11"/>
       <c r="K36" s="15">
-        <v>46097</v>
+        <v>46094</v>
       </c>
       <c r="L36" s="13" t="s">
-        <v>125</v>
-      </c>
-      <c r="M36" s="18"/>
+        <v>128</v>
+      </c>
+      <c r="M36" s="18" t="s">
+        <v>129</v>
+      </c>
       <c r="N36" s="13"/>
     </row>
     <row r="37" spans="1:14" ht="12.75">
       <c r="A37" s="11">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B37" s="11"/>
-      <c r="C37" s="12"/>
-      <c r="D37" s="13"/>
-      <c r="E37" s="13"/>
-      <c r="F37" s="13"/>
+      <c r="C37" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="D37" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="E37" s="13">
+        <v>4</v>
+      </c>
+      <c r="F37" s="13">
+        <v>5</v>
+      </c>
       <c r="G37" s="14">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H37" s="11"/>
+        <f>E37*F37</f>
+        <v>20</v>
+      </c>
+      <c r="H37" s="11" t="s">
+        <v>27</v>
+      </c>
       <c r="I37" s="13"/>
       <c r="J37" s="11"/>
-      <c r="K37" s="15"/>
-      <c r="L37" s="13"/>
-      <c r="M37" s="18"/>
+      <c r="K37" s="15">
+        <v>46097</v>
+      </c>
+      <c r="L37" s="13" t="s">
+        <v>125</v>
+      </c>
+      <c r="M37" s="17"/>
       <c r="N37" s="13"/>
     </row>
-    <row r="38" spans="1:14" ht="12.75">
-      <c r="A38" s="10">
+    <row r="38" spans="1:14" ht="60">
+      <c r="A38" s="11">
+        <v>39</v>
+      </c>
+      <c r="B38" s="13" t="s">
+        <v>131</v>
+      </c>
+      <c r="C38" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="D38" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="E38" s="13">
+        <v>2</v>
+      </c>
+      <c r="F38" s="13">
+        <v>3</v>
+      </c>
+      <c r="G38" s="13">
+        <v>6</v>
+      </c>
+      <c r="H38" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="I38" s="13" t="s">
+        <v>133</v>
+      </c>
+      <c r="J38" s="13" t="s">
+        <v>124</v>
+      </c>
+      <c r="K38" s="15">
+        <v>46101</v>
+      </c>
+      <c r="L38" s="13" t="s">
+        <v>125</v>
+      </c>
+      <c r="M38" s="18" t="s">
+        <v>134</v>
+      </c>
+      <c r="N38" s="15">
+        <v>46129</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14" ht="48" hidden="1">
+      <c r="A39" s="11">
+        <v>36</v>
+      </c>
+      <c r="B39" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="C39" s="12" t="s">
+        <v>135</v>
+      </c>
+      <c r="D39" s="34" t="s">
+        <v>26</v>
+      </c>
+      <c r="E39" s="34"/>
+      <c r="F39" s="34"/>
+      <c r="G39" s="35">
+        <f>E39*F39</f>
+        <v>0</v>
+      </c>
+      <c r="H39" s="32" t="s">
+        <v>78</v>
+      </c>
+      <c r="I39" s="34"/>
+      <c r="J39" s="32"/>
+      <c r="K39" s="19">
+        <v>46104</v>
+      </c>
+      <c r="L39" s="34" t="s">
+        <v>16</v>
+      </c>
+      <c r="M39" s="33" t="s">
+        <v>136</v>
+      </c>
+      <c r="N39" s="34"/>
+    </row>
+    <row r="40" spans="1:14" ht="96" hidden="1">
+      <c r="A40" s="10">
         <v>37</v>
       </c>
-      <c r="B38" s="11"/>
-      <c r="C38" s="12"/>
-      <c r="D38" s="13"/>
-      <c r="E38" s="13"/>
-      <c r="F38" s="13"/>
-      <c r="G38" s="14">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H38" s="11"/>
-      <c r="I38" s="13"/>
-      <c r="J38" s="11"/>
-      <c r="K38" s="15"/>
-      <c r="L38" s="13"/>
-      <c r="M38" s="18"/>
-      <c r="N38" s="13"/>
-    </row>
-    <row r="39" spans="1:14" ht="12.75">
-      <c r="A39" s="11">
-        <v>38</v>
-      </c>
-      <c r="B39" s="11"/>
-      <c r="C39" s="12"/>
-      <c r="D39" s="13"/>
-      <c r="E39" s="13"/>
-      <c r="F39" s="13"/>
-      <c r="G39" s="14">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H39" s="11"/>
-      <c r="I39" s="13"/>
-      <c r="J39" s="11"/>
-      <c r="K39" s="15"/>
-      <c r="L39" s="13"/>
-      <c r="M39" s="18"/>
-      <c r="N39" s="13"/>
-    </row>
-    <row r="40" spans="1:14" ht="12.75">
-      <c r="A40" s="11">
-        <v>39</v>
-      </c>
-      <c r="B40" s="11"/>
-      <c r="C40" s="12"/>
-      <c r="D40" s="13"/>
-      <c r="E40" s="13"/>
-      <c r="F40" s="13"/>
+      <c r="B40" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C40" s="18" t="s">
+        <v>137</v>
+      </c>
+      <c r="D40" s="13" t="s">
+        <v>138</v>
+      </c>
+      <c r="E40" s="13">
+        <v>2</v>
+      </c>
+      <c r="F40" s="13">
+        <v>2</v>
+      </c>
       <c r="G40" s="14">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H40" s="11"/>
-      <c r="I40" s="13"/>
+        <f>E40*F40</f>
+        <v>4</v>
+      </c>
+      <c r="H40" s="32" t="s">
+        <v>78</v>
+      </c>
+      <c r="I40" s="12" t="s">
+        <v>139</v>
+      </c>
       <c r="J40" s="11"/>
-      <c r="K40" s="15"/>
-      <c r="L40" s="13"/>
-      <c r="M40" s="18"/>
+      <c r="K40" s="15">
+        <v>46105</v>
+      </c>
+      <c r="L40" s="34" t="s">
+        <v>31</v>
+      </c>
+      <c r="M40" s="13"/>
       <c r="N40" s="13"/>
     </row>
-    <row r="41" spans="1:14" ht="12.75">
+    <row r="41" spans="1:14" ht="12.75" hidden="1">
       <c r="A41" s="11">
         <v>40</v>
       </c>
-      <c r="B41" s="11"/>
-      <c r="C41" s="12"/>
-      <c r="D41" s="13"/>
+      <c r="B41" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="C41" s="12" t="s">
+        <v>140</v>
+      </c>
+      <c r="D41" s="13" t="s">
+        <v>141</v>
+      </c>
       <c r="E41" s="13"/>
       <c r="F41" s="13"/>
       <c r="G41" s="14">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H41" s="11"/>
-      <c r="I41" s="13"/>
+        <f>E41*F41</f>
+        <v>0</v>
+      </c>
+      <c r="H41" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="I41" s="16" t="s">
+        <v>142</v>
+      </c>
       <c r="J41" s="11"/>
-      <c r="K41" s="15"/>
-      <c r="L41" s="13"/>
-      <c r="M41" s="18"/>
-      <c r="N41" s="13"/>
-    </row>
-    <row r="42" spans="1:14" ht="12.75">
+      <c r="K41" s="15">
+        <v>46125</v>
+      </c>
+      <c r="L41" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="M41" s="17" t="s">
+        <v>143</v>
+      </c>
+      <c r="N41" s="15">
+        <v>46125</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14" ht="12.75" hidden="1">
       <c r="A42" s="11">
         <v>41</v>
       </c>
-      <c r="B42" s="11"/>
-      <c r="C42" s="12"/>
-      <c r="D42" s="13"/>
+      <c r="B42" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="C42" s="12" t="s">
+        <v>144</v>
+      </c>
+      <c r="D42" s="13" t="s">
+        <v>141</v>
+      </c>
       <c r="E42" s="13"/>
       <c r="F42" s="13"/>
       <c r="G42" s="14">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H42" s="11"/>
-      <c r="I42" s="13"/>
+        <f>E42*F42</f>
+        <v>0</v>
+      </c>
+      <c r="H42" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="I42" s="16" t="s">
+        <v>142</v>
+      </c>
       <c r="J42" s="11"/>
-      <c r="K42" s="15"/>
-      <c r="L42" s="13"/>
-      <c r="M42" s="18"/>
-      <c r="N42" s="13"/>
-    </row>
-    <row r="43" spans="1:14" ht="12.75">
+      <c r="K42" s="15">
+        <v>46125</v>
+      </c>
+      <c r="L42" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="M42" s="17" t="s">
+        <v>143</v>
+      </c>
+      <c r="N42" s="15">
+        <v>46125</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14" ht="12.75" hidden="1">
       <c r="A43" s="11">
         <v>42</v>
       </c>
-      <c r="B43" s="11"/>
-      <c r="C43" s="12"/>
-      <c r="D43" s="13"/>
+      <c r="B43" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="C43" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="D43" s="13" t="s">
+        <v>141</v>
+      </c>
       <c r="E43" s="13"/>
       <c r="F43" s="13"/>
       <c r="G43" s="14">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H43" s="11"/>
-      <c r="I43" s="13"/>
+        <f>E43*F43</f>
+        <v>0</v>
+      </c>
+      <c r="H43" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="I43" s="16" t="s">
+        <v>142</v>
+      </c>
       <c r="J43" s="11"/>
-      <c r="K43" s="15"/>
-      <c r="L43" s="13"/>
-      <c r="M43" s="18"/>
-      <c r="N43" s="13"/>
-    </row>
-    <row r="44" spans="1:14" ht="12.75">
+      <c r="K43" s="15">
+        <v>46125</v>
+      </c>
+      <c r="L43" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="M43" s="17" t="s">
+        <v>146</v>
+      </c>
+      <c r="N43" s="15">
+        <v>46125</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14" ht="12.75" hidden="1">
       <c r="A44" s="11">
         <v>43</v>
       </c>
-      <c r="B44" s="11"/>
-      <c r="C44" s="12"/>
-      <c r="D44" s="13"/>
+      <c r="B44" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="C44" s="12" t="s">
+        <v>147</v>
+      </c>
+      <c r="D44" s="13" t="s">
+        <v>141</v>
+      </c>
       <c r="E44" s="13"/>
       <c r="F44" s="13"/>
       <c r="G44" s="14">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H44" s="11"/>
-      <c r="I44" s="13"/>
+        <f>E44*F44</f>
+        <v>0</v>
+      </c>
+      <c r="H44" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="I44" s="16" t="s">
+        <v>142</v>
+      </c>
       <c r="J44" s="11"/>
-      <c r="K44" s="15"/>
-      <c r="L44" s="13"/>
-      <c r="M44" s="18"/>
-      <c r="N44" s="13"/>
-    </row>
-    <row r="45" spans="1:14" ht="12.75">
+      <c r="K44" s="15">
+        <v>46125</v>
+      </c>
+      <c r="L44" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="M44" s="17" t="s">
+        <v>146</v>
+      </c>
+      <c r="N44" s="15">
+        <v>46125</v>
+      </c>
+    </row>
+    <row r="45" spans="1:14" ht="12.75" hidden="1">
       <c r="A45" s="10">
         <v>44</v>
       </c>
-      <c r="B45" s="11"/>
-      <c r="C45" s="12"/>
-      <c r="D45" s="13"/>
+      <c r="B45" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="C45" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="D45" s="13" t="s">
+        <v>141</v>
+      </c>
       <c r="E45" s="13"/>
       <c r="F45" s="13"/>
       <c r="G45" s="14">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H45" s="11"/>
-      <c r="I45" s="13"/>
+        <f>E45*F45</f>
+        <v>0</v>
+      </c>
+      <c r="H45" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="I45" s="16" t="s">
+        <v>142</v>
+      </c>
       <c r="J45" s="11"/>
-      <c r="K45" s="15"/>
-      <c r="L45" s="13"/>
-      <c r="M45" s="18"/>
-      <c r="N45" s="13"/>
-    </row>
-    <row r="46" spans="1:14" ht="12.75">
+      <c r="K45" s="15">
+        <v>46125</v>
+      </c>
+      <c r="L45" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="M45" s="17" t="s">
+        <v>149</v>
+      </c>
+      <c r="N45" s="15">
+        <v>46125</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14" ht="12.75" hidden="1">
       <c r="A46" s="11">
         <v>45</v>
       </c>
-      <c r="B46" s="11"/>
-      <c r="C46" s="12"/>
-      <c r="D46" s="13"/>
+      <c r="B46" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="C46" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="D46" s="13" t="s">
+        <v>141</v>
+      </c>
       <c r="E46" s="13"/>
       <c r="F46" s="13"/>
       <c r="G46" s="14">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H46" s="11"/>
-      <c r="I46" s="13"/>
+        <f>E46*F46</f>
+        <v>0</v>
+      </c>
+      <c r="H46" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="I46" s="16" t="s">
+        <v>142</v>
+      </c>
       <c r="J46" s="11"/>
-      <c r="K46" s="15"/>
-      <c r="L46" s="13"/>
-      <c r="M46" s="18"/>
-      <c r="N46" s="13"/>
-    </row>
-    <row r="47" spans="1:14" ht="12.75">
+      <c r="K46" s="15">
+        <v>46125</v>
+      </c>
+      <c r="L46" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="M46" s="17" t="s">
+        <v>151</v>
+      </c>
+      <c r="N46" s="15">
+        <v>46125</v>
+      </c>
+    </row>
+    <row r="47" spans="1:14" ht="12.75" hidden="1">
       <c r="A47" s="11">
         <v>46</v>
       </c>
-      <c r="B47" s="11"/>
-      <c r="C47" s="12"/>
-      <c r="D47" s="13"/>
+      <c r="B47" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="C47" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="D47" s="13" t="s">
+        <v>141</v>
+      </c>
       <c r="E47" s="13"/>
       <c r="F47" s="13"/>
       <c r="G47" s="14">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H47" s="11"/>
-      <c r="I47" s="13"/>
+        <f>E47*F47</f>
+        <v>0</v>
+      </c>
+      <c r="H47" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="I47" s="16" t="s">
+        <v>142</v>
+      </c>
       <c r="J47" s="11"/>
-      <c r="K47" s="15"/>
-      <c r="L47" s="13"/>
-      <c r="M47" s="18"/>
-      <c r="N47" s="13"/>
-    </row>
-    <row r="48" spans="1:14" ht="12.75">
+      <c r="K47" s="15">
+        <v>46125</v>
+      </c>
+      <c r="L47" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="M47" s="17" t="s">
+        <v>153</v>
+      </c>
+      <c r="N47" s="15">
+        <v>46125</v>
+      </c>
+    </row>
+    <row r="48" spans="1:14" ht="12.75" hidden="1">
       <c r="A48" s="11">
         <v>47</v>
       </c>
-      <c r="B48" s="11"/>
-      <c r="C48" s="12"/>
-      <c r="D48" s="13"/>
+      <c r="B48" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="C48" s="12" t="s">
+        <v>154</v>
+      </c>
+      <c r="D48" s="13" t="s">
+        <v>141</v>
+      </c>
       <c r="E48" s="13"/>
       <c r="F48" s="13"/>
       <c r="G48" s="14">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H48" s="11"/>
-      <c r="I48" s="13"/>
+        <f>E48*F48</f>
+        <v>0</v>
+      </c>
+      <c r="H48" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="I48" s="16" t="s">
+        <v>142</v>
+      </c>
       <c r="J48" s="11"/>
-      <c r="K48" s="15"/>
-      <c r="L48" s="13"/>
-      <c r="M48" s="18"/>
-      <c r="N48" s="13"/>
-    </row>
-    <row r="49" spans="1:14" ht="12.75">
+      <c r="K48" s="15">
+        <v>46125</v>
+      </c>
+      <c r="L48" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="M48" s="17" t="s">
+        <v>153</v>
+      </c>
+      <c r="N48" s="15">
+        <v>46125</v>
+      </c>
+    </row>
+    <row r="49" spans="1:14" ht="12.75" hidden="1">
       <c r="A49" s="11">
         <v>48</v>
       </c>
-      <c r="B49" s="11"/>
-      <c r="C49" s="12"/>
-      <c r="D49" s="13"/>
+      <c r="B49" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="C49" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="D49" s="13" t="s">
+        <v>141</v>
+      </c>
       <c r="E49" s="13"/>
       <c r="F49" s="13"/>
       <c r="G49" s="14">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H49" s="11"/>
-      <c r="I49" s="13"/>
+        <f>E49*F49</f>
+        <v>0</v>
+      </c>
+      <c r="H49" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="I49" s="16" t="s">
+        <v>142</v>
+      </c>
       <c r="J49" s="11"/>
-      <c r="K49" s="15"/>
-      <c r="L49" s="13"/>
-      <c r="M49" s="18"/>
-      <c r="N49" s="13"/>
-    </row>
-    <row r="50" spans="1:14" ht="12.75">
+      <c r="K49" s="15">
+        <v>46125</v>
+      </c>
+      <c r="L49" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="M49" s="17" t="s">
+        <v>153</v>
+      </c>
+      <c r="N49" s="15">
+        <v>46125</v>
+      </c>
+    </row>
+    <row r="50" spans="1:14" ht="12.75" hidden="1">
       <c r="A50" s="11">
         <v>49</v>
       </c>
-      <c r="B50" s="11"/>
-      <c r="C50" s="12"/>
-      <c r="D50" s="13"/>
+      <c r="B50" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="C50" s="12" t="s">
+        <v>156</v>
+      </c>
+      <c r="D50" s="13" t="s">
+        <v>141</v>
+      </c>
       <c r="E50" s="13"/>
       <c r="F50" s="13"/>
       <c r="G50" s="14">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H50" s="11"/>
-      <c r="I50" s="13"/>
+        <f>E50*F50</f>
+        <v>0</v>
+      </c>
+      <c r="H50" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="I50" s="16" t="s">
+        <v>142</v>
+      </c>
       <c r="J50" s="11"/>
-      <c r="K50" s="15"/>
-      <c r="L50" s="13"/>
-      <c r="M50" s="18"/>
-      <c r="N50" s="13"/>
-    </row>
-    <row r="51" spans="1:14" ht="12.75">
+      <c r="K50" s="15">
+        <v>46125</v>
+      </c>
+      <c r="L50" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="M50" s="17" t="s">
+        <v>153</v>
+      </c>
+      <c r="N50" s="15">
+        <v>46125</v>
+      </c>
+    </row>
+    <row r="51" spans="1:14" ht="12.75" hidden="1">
       <c r="A51" s="11">
         <v>50</v>
       </c>
-      <c r="B51" s="11"/>
-      <c r="C51" s="12"/>
+      <c r="B51" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="C51" s="12" t="s">
+        <v>157</v>
+      </c>
       <c r="D51" s="13"/>
       <c r="E51" s="13"/>
       <c r="F51" s="13"/>
       <c r="G51" s="14">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H51" s="11"/>
-      <c r="I51" s="13"/>
-      <c r="J51" s="11"/>
-      <c r="K51" s="15"/>
-      <c r="L51" s="13"/>
-      <c r="M51" s="18"/>
+        <f>E51*F51</f>
+        <v>0</v>
+      </c>
+      <c r="H51" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="I51" s="13" t="s">
+        <v>158</v>
+      </c>
+      <c r="J51" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="K51" s="15">
+        <v>46129</v>
+      </c>
+      <c r="L51" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="M51" s="17"/>
       <c r="N51" s="13"/>
     </row>
-    <row r="52" spans="1:14" ht="12.75">
+    <row r="52" spans="1:14" ht="12.75" hidden="1">
       <c r="A52" s="10">
         <v>51</v>
       </c>
-      <c r="B52" s="11"/>
-      <c r="C52" s="12"/>
+      <c r="B52" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="C52" s="12" t="s">
+        <v>159</v>
+      </c>
       <c r="D52" s="13"/>
       <c r="E52" s="13"/>
       <c r="F52" s="13"/>
       <c r="G52" s="14">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H52" s="11"/>
-      <c r="I52" s="13"/>
+        <f>E52*F52</f>
+        <v>0</v>
+      </c>
+      <c r="H52" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="I52" s="13" t="s">
+        <v>160</v>
+      </c>
       <c r="J52" s="11"/>
-      <c r="K52" s="15"/>
-      <c r="L52" s="13"/>
-      <c r="M52" s="18"/>
+      <c r="K52" s="15">
+        <v>46129</v>
+      </c>
+      <c r="L52" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="M52" s="17"/>
       <c r="N52" s="13"/>
     </row>
-    <row r="53" spans="1:14" ht="12.75">
+    <row r="53" spans="1:14" ht="12.75" hidden="1">
       <c r="A53" s="11">
         <v>52</v>
       </c>
@@ -3040,7 +3417,7 @@
       <c r="E53" s="13"/>
       <c r="F53" s="13"/>
       <c r="G53" s="14">
-        <f t="shared" si="0"/>
+        <f>E53*F53</f>
         <v>0</v>
       </c>
       <c r="H53" s="11"/>
@@ -3048,10 +3425,10 @@
       <c r="J53" s="11"/>
       <c r="K53" s="15"/>
       <c r="L53" s="13"/>
-      <c r="M53" s="18"/>
+      <c r="M53" s="17"/>
       <c r="N53" s="13"/>
     </row>
-    <row r="54" spans="1:14" ht="12.75">
+    <row r="54" spans="1:14" ht="12.75" hidden="1">
       <c r="A54" s="11">
         <v>53</v>
       </c>
@@ -3061,7 +3438,7 @@
       <c r="E54" s="13"/>
       <c r="F54" s="13"/>
       <c r="G54" s="14">
-        <f t="shared" si="0"/>
+        <f>E54*F54</f>
         <v>0</v>
       </c>
       <c r="H54" s="11"/>
@@ -3069,10 +3446,10 @@
       <c r="J54" s="11"/>
       <c r="K54" s="15"/>
       <c r="L54" s="13"/>
-      <c r="M54" s="18"/>
+      <c r="M54" s="17"/>
       <c r="N54" s="13"/>
     </row>
-    <row r="55" spans="1:14" ht="12.75">
+    <row r="55" spans="1:14" ht="12.75" hidden="1">
       <c r="A55" s="11">
         <v>54</v>
       </c>
@@ -3082,7 +3459,7 @@
       <c r="E55" s="13"/>
       <c r="F55" s="13"/>
       <c r="G55" s="14">
-        <f t="shared" si="0"/>
+        <f>E55*F55</f>
         <v>0</v>
       </c>
       <c r="H55" s="11"/>
@@ -3090,10 +3467,10 @@
       <c r="J55" s="11"/>
       <c r="K55" s="15"/>
       <c r="L55" s="13"/>
-      <c r="M55" s="18"/>
+      <c r="M55" s="17"/>
       <c r="N55" s="13"/>
     </row>
-    <row r="56" spans="1:14" ht="12.75">
+    <row r="56" spans="1:14" ht="12.75" hidden="1">
       <c r="A56" s="11">
         <v>55</v>
       </c>
@@ -3103,7 +3480,7 @@
       <c r="E56" s="13"/>
       <c r="F56" s="13"/>
       <c r="G56" s="14">
-        <f t="shared" si="0"/>
+        <f>E56*F56</f>
         <v>0</v>
       </c>
       <c r="H56" s="11"/>
@@ -3111,10 +3488,10 @@
       <c r="J56" s="11"/>
       <c r="K56" s="15"/>
       <c r="L56" s="13"/>
-      <c r="M56" s="18"/>
+      <c r="M56" s="17"/>
       <c r="N56" s="13"/>
     </row>
-    <row r="57" spans="1:14" ht="12.75">
+    <row r="57" spans="1:14" ht="12.75" hidden="1">
       <c r="A57" s="11">
         <v>56</v>
       </c>
@@ -3124,7 +3501,7 @@
       <c r="E57" s="13"/>
       <c r="F57" s="13"/>
       <c r="G57" s="14">
-        <f t="shared" si="0"/>
+        <f>E57*F57</f>
         <v>0</v>
       </c>
       <c r="H57" s="11"/>
@@ -3132,10 +3509,10 @@
       <c r="J57" s="11"/>
       <c r="K57" s="15"/>
       <c r="L57" s="13"/>
-      <c r="M57" s="18"/>
+      <c r="M57" s="17"/>
       <c r="N57" s="13"/>
     </row>
-    <row r="58" spans="1:14" ht="12.75">
+    <row r="58" spans="1:14" ht="12.75" hidden="1">
       <c r="A58" s="11">
         <v>57</v>
       </c>
@@ -3145,7 +3522,7 @@
       <c r="E58" s="13"/>
       <c r="F58" s="13"/>
       <c r="G58" s="14">
-        <f t="shared" si="0"/>
+        <f>E58*F58</f>
         <v>0</v>
       </c>
       <c r="H58" s="11"/>
@@ -3153,10 +3530,10 @@
       <c r="J58" s="11"/>
       <c r="K58" s="15"/>
       <c r="L58" s="13"/>
-      <c r="M58" s="18"/>
+      <c r="M58" s="17"/>
       <c r="N58" s="13"/>
     </row>
-    <row r="59" spans="1:14" ht="12.75">
+    <row r="59" spans="1:14" ht="12.75" hidden="1">
       <c r="A59" s="10">
         <v>58</v>
       </c>
@@ -3166,7 +3543,7 @@
       <c r="E59" s="13"/>
       <c r="F59" s="13"/>
       <c r="G59" s="14">
-        <f t="shared" si="0"/>
+        <f>E59*F59</f>
         <v>0</v>
       </c>
       <c r="H59" s="11"/>
@@ -3174,10 +3551,10 @@
       <c r="J59" s="11"/>
       <c r="K59" s="15"/>
       <c r="L59" s="13"/>
-      <c r="M59" s="18"/>
+      <c r="M59" s="17"/>
       <c r="N59" s="13"/>
     </row>
-    <row r="60" spans="1:14" ht="12.75">
+    <row r="60" spans="1:14" ht="12.75" hidden="1">
       <c r="A60" s="11">
         <v>59</v>
       </c>
@@ -3187,7 +3564,7 @@
       <c r="E60" s="13"/>
       <c r="F60" s="13"/>
       <c r="G60" s="14">
-        <f t="shared" si="0"/>
+        <f>E60*F60</f>
         <v>0</v>
       </c>
       <c r="H60" s="11"/>
@@ -3195,10 +3572,10 @@
       <c r="J60" s="11"/>
       <c r="K60" s="15"/>
       <c r="L60" s="13"/>
-      <c r="M60" s="18"/>
+      <c r="M60" s="17"/>
       <c r="N60" s="13"/>
     </row>
-    <row r="61" spans="1:14" ht="12.75">
+    <row r="61" spans="1:14" ht="12.75" hidden="1">
       <c r="A61" s="11">
         <v>60</v>
       </c>
@@ -3208,7 +3585,7 @@
       <c r="E61" s="13"/>
       <c r="F61" s="13"/>
       <c r="G61" s="14">
-        <f t="shared" si="0"/>
+        <f>E61*F61</f>
         <v>0</v>
       </c>
       <c r="H61" s="11"/>
@@ -3216,10 +3593,10 @@
       <c r="J61" s="11"/>
       <c r="K61" s="15"/>
       <c r="L61" s="13"/>
-      <c r="M61" s="18"/>
+      <c r="M61" s="17"/>
       <c r="N61" s="13"/>
     </row>
-    <row r="62" spans="1:14" ht="12.75">
+    <row r="62" spans="1:14" ht="12.75" hidden="1">
       <c r="A62" s="11">
         <v>61</v>
       </c>
@@ -3229,7 +3606,7 @@
       <c r="E62" s="13"/>
       <c r="F62" s="13"/>
       <c r="G62" s="14">
-        <f t="shared" si="0"/>
+        <f>E62*F62</f>
         <v>0</v>
       </c>
       <c r="H62" s="11"/>
@@ -3237,10 +3614,10 @@
       <c r="J62" s="11"/>
       <c r="K62" s="15"/>
       <c r="L62" s="13"/>
-      <c r="M62" s="18"/>
+      <c r="M62" s="17"/>
       <c r="N62" s="13"/>
     </row>
-    <row r="63" spans="1:14" ht="12.75">
+    <row r="63" spans="1:14" ht="12.75" hidden="1">
       <c r="A63" s="11">
         <v>62</v>
       </c>
@@ -3250,7 +3627,7 @@
       <c r="E63" s="13"/>
       <c r="F63" s="13"/>
       <c r="G63" s="14">
-        <f t="shared" si="0"/>
+        <f>E63*F63</f>
         <v>0</v>
       </c>
       <c r="H63" s="11"/>
@@ -3258,10 +3635,10 @@
       <c r="J63" s="11"/>
       <c r="K63" s="15"/>
       <c r="L63" s="13"/>
-      <c r="M63" s="18"/>
+      <c r="M63" s="17"/>
       <c r="N63" s="13"/>
     </row>
-    <row r="64" spans="1:14" ht="12.75">
+    <row r="64" spans="1:14" ht="12.75" hidden="1">
       <c r="A64" s="11">
         <v>63</v>
       </c>
@@ -3271,7 +3648,7 @@
       <c r="E64" s="13"/>
       <c r="F64" s="13"/>
       <c r="G64" s="14">
-        <f t="shared" si="0"/>
+        <f>E64*F64</f>
         <v>0</v>
       </c>
       <c r="H64" s="11"/>
@@ -3279,10 +3656,10 @@
       <c r="J64" s="11"/>
       <c r="K64" s="15"/>
       <c r="L64" s="13"/>
-      <c r="M64" s="18"/>
+      <c r="M64" s="17"/>
       <c r="N64" s="13"/>
     </row>
-    <row r="65" spans="1:14" ht="12.75">
+    <row r="65" spans="1:14" ht="12.75" hidden="1">
       <c r="A65" s="11">
         <v>64</v>
       </c>
@@ -3292,7 +3669,7 @@
       <c r="E65" s="13"/>
       <c r="F65" s="13"/>
       <c r="G65" s="14">
-        <f t="shared" si="0"/>
+        <f>E65*F65</f>
         <v>0</v>
       </c>
       <c r="H65" s="11"/>
@@ -3300,10 +3677,10 @@
       <c r="J65" s="11"/>
       <c r="K65" s="15"/>
       <c r="L65" s="13"/>
-      <c r="M65" s="18"/>
+      <c r="M65" s="17"/>
       <c r="N65" s="13"/>
     </row>
-    <row r="66" spans="1:14" ht="12.75">
+    <row r="66" spans="1:14" ht="12.75" hidden="1">
       <c r="A66" s="10">
         <v>65</v>
       </c>
@@ -3313,7 +3690,7 @@
       <c r="E66" s="13"/>
       <c r="F66" s="13"/>
       <c r="G66" s="14">
-        <f t="shared" si="0"/>
+        <f>E66*F66</f>
         <v>0</v>
       </c>
       <c r="H66" s="11"/>
@@ -3321,10 +3698,10 @@
       <c r="J66" s="11"/>
       <c r="K66" s="15"/>
       <c r="L66" s="13"/>
-      <c r="M66" s="18"/>
+      <c r="M66" s="17"/>
       <c r="N66" s="13"/>
     </row>
-    <row r="67" spans="1:14" ht="12.75">
+    <row r="67" spans="1:14" ht="12.75" hidden="1">
       <c r="A67" s="11">
         <v>66</v>
       </c>
@@ -3334,7 +3711,7 @@
       <c r="E67" s="13"/>
       <c r="F67" s="13"/>
       <c r="G67" s="14">
-        <f t="shared" si="0"/>
+        <f>E67*F67</f>
         <v>0</v>
       </c>
       <c r="H67" s="11"/>
@@ -3342,10 +3719,10 @@
       <c r="J67" s="11"/>
       <c r="K67" s="15"/>
       <c r="L67" s="13"/>
-      <c r="M67" s="18"/>
+      <c r="M67" s="17"/>
       <c r="N67" s="13"/>
     </row>
-    <row r="68" spans="1:14" ht="12.75">
+    <row r="68" spans="1:14" ht="12.75" hidden="1">
       <c r="A68" s="11">
         <v>67</v>
       </c>
@@ -3355,7 +3732,7 @@
       <c r="E68" s="13"/>
       <c r="F68" s="13"/>
       <c r="G68" s="14">
-        <f t="shared" si="0"/>
+        <f>E68*F68</f>
         <v>0</v>
       </c>
       <c r="H68" s="11"/>
@@ -3363,10 +3740,10 @@
       <c r="J68" s="11"/>
       <c r="K68" s="15"/>
       <c r="L68" s="13"/>
-      <c r="M68" s="18"/>
+      <c r="M68" s="17"/>
       <c r="N68" s="13"/>
     </row>
-    <row r="69" spans="1:14" ht="12.75">
+    <row r="69" spans="1:14" ht="12.75" hidden="1">
       <c r="A69" s="11">
         <v>68</v>
       </c>
@@ -3376,7 +3753,7 @@
       <c r="E69" s="13"/>
       <c r="F69" s="13"/>
       <c r="G69" s="14">
-        <f t="shared" si="0"/>
+        <f>E69*F69</f>
         <v>0</v>
       </c>
       <c r="H69" s="11"/>
@@ -3384,10 +3761,10 @@
       <c r="J69" s="11"/>
       <c r="K69" s="15"/>
       <c r="L69" s="13"/>
-      <c r="M69" s="18"/>
+      <c r="M69" s="17"/>
       <c r="N69" s="13"/>
     </row>
-    <row r="70" spans="1:14" ht="12.75">
+    <row r="70" spans="1:14" ht="12.75" hidden="1">
       <c r="A70" s="11">
         <v>69</v>
       </c>
@@ -3397,7 +3774,7 @@
       <c r="E70" s="13"/>
       <c r="F70" s="13"/>
       <c r="G70" s="14">
-        <f t="shared" si="0"/>
+        <f>E70*F70</f>
         <v>0</v>
       </c>
       <c r="H70" s="11"/>
@@ -3405,10 +3782,10 @@
       <c r="J70" s="11"/>
       <c r="K70" s="15"/>
       <c r="L70" s="13"/>
-      <c r="M70" s="18"/>
+      <c r="M70" s="17"/>
       <c r="N70" s="13"/>
     </row>
-    <row r="71" spans="1:14" ht="12.75">
+    <row r="71" spans="1:14" ht="12.75" hidden="1">
       <c r="A71" s="11">
         <v>70</v>
       </c>
@@ -3418,7 +3795,7 @@
       <c r="E71" s="13"/>
       <c r="F71" s="13"/>
       <c r="G71" s="14">
-        <f t="shared" si="0"/>
+        <f>E71*F71</f>
         <v>0</v>
       </c>
       <c r="H71" s="11"/>
@@ -3426,10 +3803,10 @@
       <c r="J71" s="11"/>
       <c r="K71" s="15"/>
       <c r="L71" s="13"/>
-      <c r="M71" s="18"/>
+      <c r="M71" s="17"/>
       <c r="N71" s="13"/>
     </row>
-    <row r="72" spans="1:14" ht="12.75">
+    <row r="72" spans="1:14" ht="12.75" hidden="1">
       <c r="A72" s="11">
         <v>71</v>
       </c>
@@ -3439,7 +3816,7 @@
       <c r="E72" s="13"/>
       <c r="F72" s="13"/>
       <c r="G72" s="14">
-        <f t="shared" si="0"/>
+        <f>E72*F72</f>
         <v>0</v>
       </c>
       <c r="H72" s="11"/>
@@ -3447,10 +3824,10 @@
       <c r="J72" s="11"/>
       <c r="K72" s="15"/>
       <c r="L72" s="13"/>
-      <c r="M72" s="18"/>
+      <c r="M72" s="17"/>
       <c r="N72" s="13"/>
     </row>
-    <row r="73" spans="1:14" ht="12.75">
+    <row r="73" spans="1:14" ht="12.75" hidden="1">
       <c r="A73" s="10">
         <v>72</v>
       </c>
@@ -3460,7 +3837,7 @@
       <c r="E73" s="13"/>
       <c r="F73" s="13"/>
       <c r="G73" s="14">
-        <f t="shared" si="0"/>
+        <f>E73*F73</f>
         <v>0</v>
       </c>
       <c r="H73" s="11"/>
@@ -3468,10 +3845,10 @@
       <c r="J73" s="11"/>
       <c r="K73" s="15"/>
       <c r="L73" s="13"/>
-      <c r="M73" s="18"/>
+      <c r="M73" s="17"/>
       <c r="N73" s="13"/>
     </row>
-    <row r="74" spans="1:14" ht="12.75">
+    <row r="74" spans="1:14" ht="12.75" hidden="1">
       <c r="A74" s="11">
         <v>73</v>
       </c>
@@ -3481,7 +3858,7 @@
       <c r="E74" s="13"/>
       <c r="F74" s="13"/>
       <c r="G74" s="14">
-        <f t="shared" si="0"/>
+        <f>E74*F74</f>
         <v>0</v>
       </c>
       <c r="H74" s="11"/>
@@ -3489,10 +3866,10 @@
       <c r="J74" s="11"/>
       <c r="K74" s="15"/>
       <c r="L74" s="13"/>
-      <c r="M74" s="18"/>
+      <c r="M74" s="17"/>
       <c r="N74" s="13"/>
     </row>
-    <row r="75" spans="1:14" ht="12.75">
+    <row r="75" spans="1:14" ht="12.75" hidden="1">
       <c r="A75" s="11">
         <v>74</v>
       </c>
@@ -3502,7 +3879,7 @@
       <c r="E75" s="13"/>
       <c r="F75" s="13"/>
       <c r="G75" s="14">
-        <f t="shared" si="0"/>
+        <f>E75*F75</f>
         <v>0</v>
       </c>
       <c r="H75" s="11"/>
@@ -3510,10 +3887,10 @@
       <c r="J75" s="11"/>
       <c r="K75" s="15"/>
       <c r="L75" s="13"/>
-      <c r="M75" s="18"/>
+      <c r="M75" s="17"/>
       <c r="N75" s="13"/>
     </row>
-    <row r="76" spans="1:14" ht="12.75">
+    <row r="76" spans="1:14" ht="12.75" hidden="1">
       <c r="A76" s="11">
         <v>75</v>
       </c>
@@ -3523,7 +3900,7 @@
       <c r="E76" s="13"/>
       <c r="F76" s="13"/>
       <c r="G76" s="14">
-        <f t="shared" si="0"/>
+        <f>E76*F76</f>
         <v>0</v>
       </c>
       <c r="H76" s="11"/>
@@ -3531,10 +3908,10 @@
       <c r="J76" s="11"/>
       <c r="K76" s="15"/>
       <c r="L76" s="13"/>
-      <c r="M76" s="18"/>
+      <c r="M76" s="17"/>
       <c r="N76" s="13"/>
     </row>
-    <row r="77" spans="1:14" ht="12.75">
+    <row r="77" spans="1:14" ht="12.75" hidden="1">
       <c r="A77" s="11">
         <v>76</v>
       </c>
@@ -3544,7 +3921,7 @@
       <c r="E77" s="13"/>
       <c r="F77" s="13"/>
       <c r="G77" s="14">
-        <f t="shared" si="0"/>
+        <f>E77*F77</f>
         <v>0</v>
       </c>
       <c r="H77" s="11"/>
@@ -3552,10 +3929,10 @@
       <c r="J77" s="11"/>
       <c r="K77" s="15"/>
       <c r="L77" s="13"/>
-      <c r="M77" s="18"/>
+      <c r="M77" s="17"/>
       <c r="N77" s="13"/>
     </row>
-    <row r="78" spans="1:14" ht="12.75">
+    <row r="78" spans="1:14" ht="12.75" hidden="1">
       <c r="A78" s="11">
         <v>77</v>
       </c>
@@ -3565,7 +3942,7 @@
       <c r="E78" s="13"/>
       <c r="F78" s="13"/>
       <c r="G78" s="14">
-        <f t="shared" si="0"/>
+        <f>E78*F78</f>
         <v>0</v>
       </c>
       <c r="H78" s="11"/>
@@ -3573,10 +3950,10 @@
       <c r="J78" s="11"/>
       <c r="K78" s="15"/>
       <c r="L78" s="13"/>
-      <c r="M78" s="18"/>
+      <c r="M78" s="17"/>
       <c r="N78" s="13"/>
     </row>
-    <row r="79" spans="1:14" ht="12.75">
+    <row r="79" spans="1:14" ht="12.75" hidden="1">
       <c r="A79" s="11">
         <v>78</v>
       </c>
@@ -3586,7 +3963,7 @@
       <c r="E79" s="13"/>
       <c r="F79" s="13"/>
       <c r="G79" s="14">
-        <f t="shared" si="0"/>
+        <f>E79*F79</f>
         <v>0</v>
       </c>
       <c r="H79" s="11"/>
@@ -3594,10 +3971,10 @@
       <c r="J79" s="11"/>
       <c r="K79" s="15"/>
       <c r="L79" s="13"/>
-      <c r="M79" s="18"/>
+      <c r="M79" s="17"/>
       <c r="N79" s="13"/>
     </row>
-    <row r="80" spans="1:14" ht="12.75">
+    <row r="80" spans="1:14" ht="12.75" hidden="1">
       <c r="A80" s="10">
         <v>79</v>
       </c>
@@ -3607,7 +3984,7 @@
       <c r="E80" s="13"/>
       <c r="F80" s="13"/>
       <c r="G80" s="14">
-        <f t="shared" si="0"/>
+        <f>E80*F80</f>
         <v>0</v>
       </c>
       <c r="H80" s="11"/>
@@ -3615,10 +3992,10 @@
       <c r="J80" s="11"/>
       <c r="K80" s="15"/>
       <c r="L80" s="13"/>
-      <c r="M80" s="18"/>
+      <c r="M80" s="17"/>
       <c r="N80" s="13"/>
     </row>
-    <row r="81" spans="1:14" ht="12.75">
+    <row r="81" spans="1:14" ht="12.75" hidden="1">
       <c r="A81" s="11">
         <v>80</v>
       </c>
@@ -3628,7 +4005,7 @@
       <c r="E81" s="13"/>
       <c r="F81" s="13"/>
       <c r="G81" s="14">
-        <f t="shared" si="0"/>
+        <f>E81*F81</f>
         <v>0</v>
       </c>
       <c r="H81" s="11"/>
@@ -3636,10 +4013,10 @@
       <c r="J81" s="11"/>
       <c r="K81" s="15"/>
       <c r="L81" s="13"/>
-      <c r="M81" s="18"/>
+      <c r="M81" s="17"/>
       <c r="N81" s="13"/>
     </row>
-    <row r="82" spans="1:14" ht="12.75">
+    <row r="82" spans="1:14" ht="12.75" hidden="1">
       <c r="A82" s="11">
         <v>81</v>
       </c>
@@ -3649,7 +4026,7 @@
       <c r="E82" s="13"/>
       <c r="F82" s="13"/>
       <c r="G82" s="14">
-        <f t="shared" si="0"/>
+        <f>E82*F82</f>
         <v>0</v>
       </c>
       <c r="H82" s="11"/>
@@ -3657,10 +4034,10 @@
       <c r="J82" s="11"/>
       <c r="K82" s="15"/>
       <c r="L82" s="13"/>
-      <c r="M82" s="18"/>
+      <c r="M82" s="17"/>
       <c r="N82" s="13"/>
     </row>
-    <row r="83" spans="1:14" ht="12.75">
+    <row r="83" spans="1:14" ht="12.75" hidden="1">
       <c r="A83" s="11">
         <v>82</v>
       </c>
@@ -3670,7 +4047,7 @@
       <c r="E83" s="13"/>
       <c r="F83" s="13"/>
       <c r="G83" s="14">
-        <f t="shared" si="0"/>
+        <f>E83*F83</f>
         <v>0</v>
       </c>
       <c r="H83" s="11"/>
@@ -3678,10 +4055,10 @@
       <c r="J83" s="11"/>
       <c r="K83" s="15"/>
       <c r="L83" s="13"/>
-      <c r="M83" s="18"/>
+      <c r="M83" s="17"/>
       <c r="N83" s="13"/>
     </row>
-    <row r="84" spans="1:14" ht="12.75">
+    <row r="84" spans="1:14" ht="12.75" hidden="1">
       <c r="A84" s="11">
         <v>83</v>
       </c>
@@ -3691,7 +4068,7 @@
       <c r="E84" s="13"/>
       <c r="F84" s="13"/>
       <c r="G84" s="14">
-        <f t="shared" si="0"/>
+        <f>E84*F84</f>
         <v>0</v>
       </c>
       <c r="H84" s="11"/>
@@ -3699,10 +4076,10 @@
       <c r="J84" s="11"/>
       <c r="K84" s="15"/>
       <c r="L84" s="13"/>
-      <c r="M84" s="18"/>
+      <c r="M84" s="17"/>
       <c r="N84" s="13"/>
     </row>
-    <row r="85" spans="1:14" ht="12.75">
+    <row r="85" spans="1:14" ht="12.75" hidden="1">
       <c r="A85" s="11">
         <v>84</v>
       </c>
@@ -3712,7 +4089,7 @@
       <c r="E85" s="13"/>
       <c r="F85" s="13"/>
       <c r="G85" s="14">
-        <f t="shared" si="0"/>
+        <f>E85*F85</f>
         <v>0</v>
       </c>
       <c r="H85" s="11"/>
@@ -3720,10 +4097,10 @@
       <c r="J85" s="11"/>
       <c r="K85" s="15"/>
       <c r="L85" s="13"/>
-      <c r="M85" s="18"/>
+      <c r="M85" s="17"/>
       <c r="N85" s="13"/>
     </row>
-    <row r="86" spans="1:14" ht="12.75">
+    <row r="86" spans="1:14" ht="12.75" hidden="1">
       <c r="A86" s="11">
         <v>85</v>
       </c>
@@ -3733,7 +4110,7 @@
       <c r="E86" s="13"/>
       <c r="F86" s="13"/>
       <c r="G86" s="14">
-        <f t="shared" si="0"/>
+        <f>E86*F86</f>
         <v>0</v>
       </c>
       <c r="H86" s="11"/>
@@ -3741,10 +4118,10 @@
       <c r="J86" s="11"/>
       <c r="K86" s="15"/>
       <c r="L86" s="13"/>
-      <c r="M86" s="18"/>
+      <c r="M86" s="17"/>
       <c r="N86" s="13"/>
     </row>
-    <row r="87" spans="1:14" ht="12.75">
+    <row r="87" spans="1:14" ht="12.75" hidden="1">
       <c r="A87" s="10">
         <v>86</v>
       </c>
@@ -3754,7 +4131,7 @@
       <c r="E87" s="13"/>
       <c r="F87" s="13"/>
       <c r="G87" s="14">
-        <f t="shared" si="0"/>
+        <f>E87*F87</f>
         <v>0</v>
       </c>
       <c r="H87" s="11"/>
@@ -3762,10 +4139,10 @@
       <c r="J87" s="11"/>
       <c r="K87" s="15"/>
       <c r="L87" s="13"/>
-      <c r="M87" s="18"/>
+      <c r="M87" s="17"/>
       <c r="N87" s="13"/>
     </row>
-    <row r="88" spans="1:14" ht="12.75">
+    <row r="88" spans="1:14" ht="12.75" hidden="1">
       <c r="A88" s="11">
         <v>87</v>
       </c>
@@ -3775,7 +4152,7 @@
       <c r="E88" s="13"/>
       <c r="F88" s="13"/>
       <c r="G88" s="14">
-        <f t="shared" si="0"/>
+        <f>E88*F88</f>
         <v>0</v>
       </c>
       <c r="H88" s="11"/>
@@ -3783,10 +4160,10 @@
       <c r="J88" s="11"/>
       <c r="K88" s="15"/>
       <c r="L88" s="13"/>
-      <c r="M88" s="18"/>
+      <c r="M88" s="17"/>
       <c r="N88" s="13"/>
     </row>
-    <row r="89" spans="1:14" ht="12.75">
+    <row r="89" spans="1:14" ht="12.75" hidden="1">
       <c r="A89" s="11">
         <v>88</v>
       </c>
@@ -3796,7 +4173,7 @@
       <c r="E89" s="13"/>
       <c r="F89" s="13"/>
       <c r="G89" s="14">
-        <f t="shared" si="0"/>
+        <f>E89*F89</f>
         <v>0</v>
       </c>
       <c r="H89" s="11"/>
@@ -3804,10 +4181,10 @@
       <c r="J89" s="11"/>
       <c r="K89" s="15"/>
       <c r="L89" s="13"/>
-      <c r="M89" s="18"/>
+      <c r="M89" s="17"/>
       <c r="N89" s="13"/>
     </row>
-    <row r="90" spans="1:14" ht="12.75">
+    <row r="90" spans="1:14" ht="12.75" hidden="1">
       <c r="A90" s="11">
         <v>89</v>
       </c>
@@ -3817,7 +4194,7 @@
       <c r="E90" s="13"/>
       <c r="F90" s="13"/>
       <c r="G90" s="14">
-        <f t="shared" si="0"/>
+        <f>E90*F90</f>
         <v>0</v>
       </c>
       <c r="H90" s="11"/>
@@ -3825,10 +4202,10 @@
       <c r="J90" s="11"/>
       <c r="K90" s="15"/>
       <c r="L90" s="13"/>
-      <c r="M90" s="18"/>
+      <c r="M90" s="17"/>
       <c r="N90" s="13"/>
     </row>
-    <row r="91" spans="1:14" ht="12.75">
+    <row r="91" spans="1:14" ht="12.75" hidden="1">
       <c r="A91" s="11">
         <v>90</v>
       </c>
@@ -3838,7 +4215,7 @@
       <c r="E91" s="13"/>
       <c r="F91" s="13"/>
       <c r="G91" s="14">
-        <f t="shared" si="0"/>
+        <f>E91*F91</f>
         <v>0</v>
       </c>
       <c r="H91" s="11"/>
@@ -3846,10 +4223,10 @@
       <c r="J91" s="11"/>
       <c r="K91" s="15"/>
       <c r="L91" s="13"/>
-      <c r="M91" s="18"/>
+      <c r="M91" s="17"/>
       <c r="N91" s="13"/>
     </row>
-    <row r="92" spans="1:14" ht="12.75">
+    <row r="92" spans="1:14" ht="12.75" hidden="1">
       <c r="A92" s="11">
         <v>91</v>
       </c>
@@ -3859,7 +4236,7 @@
       <c r="E92" s="13"/>
       <c r="F92" s="13"/>
       <c r="G92" s="14">
-        <f t="shared" si="0"/>
+        <f>E92*F92</f>
         <v>0</v>
       </c>
       <c r="H92" s="11"/>
@@ -3867,10 +4244,10 @@
       <c r="J92" s="11"/>
       <c r="K92" s="15"/>
       <c r="L92" s="13"/>
-      <c r="M92" s="18"/>
+      <c r="M92" s="17"/>
       <c r="N92" s="13"/>
     </row>
-    <row r="93" spans="1:14" ht="12.75">
+    <row r="93" spans="1:14" ht="12.75" hidden="1">
       <c r="A93" s="11">
         <v>92</v>
       </c>
@@ -3880,7 +4257,7 @@
       <c r="E93" s="13"/>
       <c r="F93" s="13"/>
       <c r="G93" s="14">
-        <f t="shared" si="0"/>
+        <f>E93*F93</f>
         <v>0</v>
       </c>
       <c r="H93" s="11"/>
@@ -3888,10 +4265,10 @@
       <c r="J93" s="11"/>
       <c r="K93" s="15"/>
       <c r="L93" s="13"/>
-      <c r="M93" s="18"/>
+      <c r="M93" s="17"/>
       <c r="N93" s="13"/>
     </row>
-    <row r="94" spans="1:14" ht="12.75">
+    <row r="94" spans="1:14" ht="12.75" hidden="1">
       <c r="A94" s="10">
         <v>93</v>
       </c>
@@ -3901,7 +4278,7 @@
       <c r="E94" s="13"/>
       <c r="F94" s="13"/>
       <c r="G94" s="14">
-        <f t="shared" si="0"/>
+        <f>E94*F94</f>
         <v>0</v>
       </c>
       <c r="H94" s="11"/>
@@ -3909,10 +4286,10 @@
       <c r="J94" s="11"/>
       <c r="K94" s="15"/>
       <c r="L94" s="13"/>
-      <c r="M94" s="18"/>
+      <c r="M94" s="17"/>
       <c r="N94" s="13"/>
     </row>
-    <row r="95" spans="1:14" ht="12.75">
+    <row r="95" spans="1:14" ht="12.75" hidden="1">
       <c r="A95" s="11">
         <v>94</v>
       </c>
@@ -3922,7 +4299,7 @@
       <c r="E95" s="13"/>
       <c r="F95" s="13"/>
       <c r="G95" s="14">
-        <f t="shared" si="0"/>
+        <f>E95*F95</f>
         <v>0</v>
       </c>
       <c r="H95" s="11"/>
@@ -3930,10 +4307,10 @@
       <c r="J95" s="11"/>
       <c r="K95" s="15"/>
       <c r="L95" s="13"/>
-      <c r="M95" s="18"/>
+      <c r="M95" s="17"/>
       <c r="N95" s="13"/>
     </row>
-    <row r="96" spans="1:14" ht="12.75">
+    <row r="96" spans="1:14" ht="12.75" hidden="1">
       <c r="A96" s="11">
         <v>95</v>
       </c>
@@ -3943,7 +4320,7 @@
       <c r="E96" s="13"/>
       <c r="F96" s="13"/>
       <c r="G96" s="14">
-        <f t="shared" si="0"/>
+        <f>E96*F96</f>
         <v>0</v>
       </c>
       <c r="H96" s="11"/>
@@ -3951,10 +4328,10 @@
       <c r="J96" s="11"/>
       <c r="K96" s="15"/>
       <c r="L96" s="13"/>
-      <c r="M96" s="18"/>
+      <c r="M96" s="17"/>
       <c r="N96" s="13"/>
     </row>
-    <row r="97" spans="1:14" ht="12.75">
+    <row r="97" spans="1:14" ht="12.75" hidden="1">
       <c r="A97" s="11">
         <v>96</v>
       </c>
@@ -3964,7 +4341,7 @@
       <c r="E97" s="13"/>
       <c r="F97" s="13"/>
       <c r="G97" s="14">
-        <f t="shared" si="0"/>
+        <f>E97*F97</f>
         <v>0</v>
       </c>
       <c r="H97" s="11"/>
@@ -3972,10 +4349,10 @@
       <c r="J97" s="11"/>
       <c r="K97" s="15"/>
       <c r="L97" s="13"/>
-      <c r="M97" s="18"/>
+      <c r="M97" s="17"/>
       <c r="N97" s="13"/>
     </row>
-    <row r="98" spans="1:14" ht="12.75">
+    <row r="98" spans="1:14" ht="12.75" hidden="1">
       <c r="A98" s="11">
         <v>97</v>
       </c>
@@ -3985,7 +4362,7 @@
       <c r="E98" s="13"/>
       <c r="F98" s="13"/>
       <c r="G98" s="14">
-        <f t="shared" si="0"/>
+        <f>E98*F98</f>
         <v>0</v>
       </c>
       <c r="H98" s="11"/>
@@ -3993,10 +4370,10 @@
       <c r="J98" s="11"/>
       <c r="K98" s="15"/>
       <c r="L98" s="13"/>
-      <c r="M98" s="18"/>
+      <c r="M98" s="17"/>
       <c r="N98" s="13"/>
     </row>
-    <row r="99" spans="1:14" ht="12.75">
+    <row r="99" spans="1:14" ht="12.75" hidden="1">
       <c r="A99" s="11">
         <v>98</v>
       </c>
@@ -4006,7 +4383,7 @@
       <c r="E99" s="13"/>
       <c r="F99" s="13"/>
       <c r="G99" s="14">
-        <f t="shared" si="0"/>
+        <f>E99*F99</f>
         <v>0</v>
       </c>
       <c r="H99" s="11"/>
@@ -4014,10 +4391,10 @@
       <c r="J99" s="11"/>
       <c r="K99" s="15"/>
       <c r="L99" s="13"/>
-      <c r="M99" s="18"/>
+      <c r="M99" s="17"/>
       <c r="N99" s="13"/>
     </row>
-    <row r="100" spans="1:14" ht="12.75">
+    <row r="100" spans="1:14" ht="12.75" hidden="1">
       <c r="A100" s="11">
         <v>99</v>
       </c>
@@ -4027,7 +4404,7 @@
       <c r="E100" s="13"/>
       <c r="F100" s="13"/>
       <c r="G100" s="14">
-        <f t="shared" si="0"/>
+        <f>E100*F100</f>
         <v>0</v>
       </c>
       <c r="H100" s="11"/>
@@ -4035,72 +4412,48 @@
       <c r="J100" s="11"/>
       <c r="K100" s="15"/>
       <c r="L100" s="13"/>
-      <c r="M100" s="18"/>
+      <c r="M100" s="17"/>
       <c r="N100" s="13"/>
     </row>
-    <row r="101" spans="1:14" ht="12.75">
-      <c r="A101" s="33">
+    <row r="101" spans="1:14" ht="12.75" hidden="1">
+      <c r="A101" s="31">
         <v>100</v>
       </c>
-      <c r="B101" s="34"/>
-      <c r="C101" s="35"/>
-      <c r="D101" s="36"/>
-      <c r="E101" s="36"/>
-      <c r="F101" s="36"/>
-      <c r="G101" s="37">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H101" s="34"/>
-      <c r="I101" s="36"/>
-      <c r="J101" s="34"/>
-      <c r="K101" s="20"/>
-      <c r="L101" s="36"/>
-      <c r="M101" s="23"/>
-      <c r="N101" s="36"/>
-    </row>
-    <row r="102" spans="1:14" ht="24">
-      <c r="A102" s="13">
-        <v>30</v>
-      </c>
-      <c r="B102" s="13" t="s">
-        <v>126</v>
-      </c>
-      <c r="C102" s="12" t="s">
-        <v>127</v>
-      </c>
-      <c r="D102" s="36" t="s">
-        <v>69</v>
-      </c>
-      <c r="E102" s="36">
-        <v>5</v>
-      </c>
-      <c r="F102" s="36">
-        <v>5</v>
-      </c>
-      <c r="G102" s="36">
-        <v>25</v>
-      </c>
-      <c r="H102" s="36" t="s">
-        <v>35</v>
-      </c>
-      <c r="I102" s="36" t="s">
-        <v>128</v>
-      </c>
-      <c r="J102" s="36"/>
-      <c r="K102" s="20">
-        <v>46093</v>
-      </c>
-      <c r="L102" s="36" t="s">
-        <v>125</v>
-      </c>
-      <c r="M102" s="36" t="s">
-        <v>129</v>
-      </c>
-      <c r="N102" s="36"/>
+      <c r="B101" s="32"/>
+      <c r="C101" s="33"/>
+      <c r="D101" s="34"/>
+      <c r="E101" s="34"/>
+      <c r="F101" s="34"/>
+      <c r="G101" s="35">
+        <f>E101*F101</f>
+        <v>0</v>
+      </c>
+      <c r="H101" s="32"/>
+      <c r="I101" s="34"/>
+      <c r="J101" s="32"/>
+      <c r="K101" s="19"/>
+      <c r="L101" s="34"/>
+      <c r="M101" s="21"/>
+      <c r="N101" s="34"/>
+    </row>
+    <row r="102" spans="1:14" ht="12.75">
+      <c r="A102" s="13"/>
+      <c r="B102" s="13"/>
+      <c r="C102" s="12"/>
+      <c r="D102" s="34"/>
+      <c r="E102" s="34"/>
+      <c r="F102" s="34"/>
+      <c r="G102" s="34"/>
+      <c r="H102" s="34"/>
+      <c r="I102" s="34"/>
+      <c r="J102" s="34"/>
+      <c r="K102" s="19"/>
+      <c r="L102" s="34"/>
+      <c r="M102" s="34"/>
+      <c r="N102" s="34"/>
     </row>
     <row r="103" spans="1:14" ht="12.75">
-      <c r="C103" s="19"/>
+      <c r="C103" s="18"/>
       <c r="D103" s="12"/>
       <c r="E103" s="13"/>
       <c r="F103" s="13"/>
@@ -4114,14 +4467,32 @@
       <c r="N103" s="13"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Z103" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:Z101" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="7">
+      <filters>
+        <filter val="In Progress"/>
+      </filters>
+    </filterColumn>
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:Z101">
+      <sortCondition ref="N1:N101"/>
+    </sortState>
+  </autoFilter>
   <hyperlinks>
     <hyperlink ref="J14" r:id="rId1" display="https://oncologyanalyticsinc-my.sharepoint.com/:w:/r/personal/jhall_oncologyanalytics_com/_layouts/15/Doc.aspx?sourcedoc=%7B447717B2-BE52-4C47-AE81-AD9FCC38A4A6%7D&amp;file=Automapper%20or%20No.docx&amp;action=default&amp;mobileredirect=true&amp;DefaultItemOpen=1&amp;wdOrigin=WAC.WORD.HOME-BUTTON%2CAPPHOME-WEB.FILEBROWSER.RECENT&amp;wdPreviousSession=ebc71ebf-660e-45eb-a477-b52e302885d9&amp;wdPreviousSessionSrc=AppHomeWeb&amp;ct=1769183354671" xr:uid="{4538ABC9-487B-4F26-B2E6-EB005E194DA6}"/>
-    <hyperlink ref="J20" r:id="rId2" xr:uid="{3CE0B1D6-148B-48AF-BF32-D0DEE37B825C}"/>
-    <hyperlink ref="M33" r:id="rId3" xr:uid="{A29F51EE-575A-4E3E-9302-0B5F9B18E4BE}"/>
+    <hyperlink ref="I20" r:id="rId2" xr:uid="{3CE0B1D6-148B-48AF-BF32-D0DEE37B825C}"/>
+    <hyperlink ref="I41" r:id="rId3" xr:uid="{8E24C642-3972-4317-B719-3015D4520588}"/>
+    <hyperlink ref="I42" r:id="rId4" xr:uid="{C78EB14B-E6C0-4F93-93AD-6CCAC77E93F0}"/>
+    <hyperlink ref="I43" r:id="rId5" xr:uid="{5197C272-CF70-467C-A214-BBDD4981881C}"/>
+    <hyperlink ref="I44" r:id="rId6" xr:uid="{25E67BA4-6572-4CED-ABB6-7789F15B08BD}"/>
+    <hyperlink ref="I45" r:id="rId7" xr:uid="{FAC7063D-B680-44E5-831C-3610823A73A0}"/>
+    <hyperlink ref="I46" r:id="rId8" xr:uid="{7D40AE2B-38AA-46B0-B52C-6CD6E05D4AA2}"/>
+    <hyperlink ref="I47" r:id="rId9" xr:uid="{F772FA5F-0773-4E5F-81FF-855B82651035}"/>
+    <hyperlink ref="I48" r:id="rId10" xr:uid="{D9ECB439-CEE2-42B0-BCDF-21D2188CB724}"/>
+    <hyperlink ref="I49" r:id="rId11" xr:uid="{18E8CE66-BF04-440F-949C-06178D16FAD3}"/>
+    <hyperlink ref="I50" r:id="rId12" xr:uid="{07A19021-8D16-4AEC-B9AF-F28A5A9A8317}"/>
   </hyperlinks>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-  <legacyDrawing r:id="rId4"/>
+  <legacyDrawing r:id="rId13"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
@@ -4129,19 +4500,19 @@
           <x14:formula1>
             <xm:f>Definitions!$B$40:$B$43</xm:f>
           </x14:formula1>
-          <xm:sqref>B2:B101</xm:sqref>
+          <xm:sqref>B2:B38 B41:B101</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000001000000}">
           <x14:formula1>
             <xm:f>Definitions!$B$28:$B$31</xm:f>
           </x14:formula1>
-          <xm:sqref>H2:H101</xm:sqref>
+          <xm:sqref>H2:H38 H41:H101</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000002000000}">
           <x14:formula1>
             <xm:f>Definitions!$B$34:$B$37</xm:f>
           </x14:formula1>
-          <xm:sqref>J21:J101 J2:J19</xm:sqref>
+          <xm:sqref>J21:J38 J7:J19 I6 J2:J5 J41:J101</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -4154,89 +4525,89 @@
   <dimension ref="A1:I7"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
-    <col min="1" max="1" width="18.28515625" style="25" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17" style="25" customWidth="1"/>
-    <col min="3" max="3" width="23.140625" style="25" customWidth="1"/>
-    <col min="4" max="4" width="17.42578125" style="26" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.7109375" style="26" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.28515625" style="23" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17" style="23" customWidth="1"/>
+    <col min="3" max="3" width="23.140625" style="23" customWidth="1"/>
+    <col min="4" max="4" width="17.42578125" style="24" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.7109375" style="24" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.7109375" style="32" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.7109375" style="27" customWidth="1"/>
+    <col min="7" max="7" width="16.7109375" style="30" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.7109375" style="25" customWidth="1"/>
     <col min="9" max="9" width="12.85546875" style="7" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
-      <c r="A1" s="25" t="s">
-        <v>130</v>
-      </c>
-      <c r="B1" s="25" t="s">
+      <c r="A1" s="23" t="s">
+        <v>161</v>
+      </c>
+      <c r="B1" s="23" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="25" t="s">
-        <v>131</v>
-      </c>
-      <c r="D1" s="26" t="s">
-        <v>132</v>
-      </c>
-      <c r="E1" s="26" t="s">
-        <v>133</v>
+      <c r="C1" s="23" t="s">
+        <v>162</v>
+      </c>
+      <c r="D1" s="24" t="s">
+        <v>163</v>
+      </c>
+      <c r="E1" s="24" t="s">
+        <v>164</v>
       </c>
       <c r="F1" t="s">
-        <v>134</v>
-      </c>
-      <c r="G1" s="32" t="s">
-        <v>135</v>
-      </c>
-      <c r="H1" s="27" t="s">
+        <v>165</v>
+      </c>
+      <c r="G1" s="30" t="s">
+        <v>166</v>
+      </c>
+      <c r="H1" s="25" t="s">
         <v>11</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" s="29" customFormat="1" ht="24">
-      <c r="A2" s="28" t="s">
-        <v>137</v>
-      </c>
-      <c r="B2" s="28" t="s">
-        <v>138</v>
-      </c>
-      <c r="C2" s="31" t="s">
-        <v>139</v>
-      </c>
-      <c r="D2" s="27" t="s">
-        <v>69</v>
-      </c>
-      <c r="E2" s="27" t="s">
-        <v>140</v>
-      </c>
-      <c r="F2" s="27" t="s">
-        <v>141</v>
-      </c>
-      <c r="G2" s="32">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" s="27" customFormat="1" ht="24">
+      <c r="A2" s="26" t="s">
+        <v>168</v>
+      </c>
+      <c r="B2" s="26" t="s">
+        <v>169</v>
+      </c>
+      <c r="C2" s="29" t="s">
+        <v>170</v>
+      </c>
+      <c r="D2" s="25" t="s">
+        <v>68</v>
+      </c>
+      <c r="E2" s="25" t="s">
+        <v>171</v>
+      </c>
+      <c r="F2" s="25" t="s">
+        <v>172</v>
+      </c>
+      <c r="G2" s="30">
         <v>46090</v>
       </c>
-      <c r="H2" s="27" t="s">
-        <v>47</v>
-      </c>
-      <c r="I2" s="30" t="s">
-        <v>142</v>
+      <c r="H2" s="25" t="s">
+        <v>46</v>
+      </c>
+      <c r="I2" s="28" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="3" spans="1:9">
-      <c r="F3" s="26"/>
+      <c r="F3" s="24"/>
     </row>
     <row r="4" spans="1:9">
-      <c r="F4" s="26"/>
+      <c r="F4" s="24"/>
     </row>
     <row r="5" spans="1:9">
-      <c r="F5" s="26"/>
+      <c r="F5" s="24"/>
     </row>
     <row r="6" spans="1:9">
-      <c r="F6" s="26"/>
+      <c r="F6" s="24"/>
     </row>
     <row r="7" spans="1:9">
-      <c r="F7" s="26"/>
+      <c r="F7" s="24"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -4269,7 +4640,7 @@
   <sheetData>
     <row r="1" spans="1:3" ht="12.75">
       <c r="A1" s="3" t="s">
-        <v>143</v>
+        <v>174</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="12.75">
@@ -4277,15 +4648,15 @@
     </row>
     <row r="3" spans="1:3" ht="12.75">
       <c r="A3" s="4" t="s">
-        <v>144</v>
+        <v>175</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="12.75">
       <c r="A4" s="3" t="s">
-        <v>145</v>
+        <v>176</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>146</v>
+        <v>177</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>2</v>
@@ -4296,10 +4667,10 @@
         <v>5</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>147</v>
+        <v>178</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>148</v>
+        <v>179</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="12.75">
@@ -4307,10 +4678,10 @@
         <v>4</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>149</v>
+        <v>180</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>150</v>
+        <v>181</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="12.75">
@@ -4318,10 +4689,10 @@
         <v>3</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>151</v>
+        <v>182</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>152</v>
+        <v>183</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="12.75">
@@ -4329,10 +4700,10 @@
         <v>2</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>153</v>
+        <v>184</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>154</v>
+        <v>185</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="12.75">
@@ -4340,23 +4711,23 @@
         <v>1</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>155</v>
+        <v>186</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>156</v>
+        <v>187</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="12.75">
       <c r="A12" s="4" t="s">
-        <v>157</v>
+        <v>188</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="12.75">
       <c r="A13" s="3" t="s">
-        <v>145</v>
+        <v>176</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>146</v>
+        <v>177</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>2</v>
@@ -4367,10 +4738,10 @@
         <v>5</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>158</v>
+        <v>189</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>159</v>
+        <v>190</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="12.75">
@@ -4378,10 +4749,10 @@
         <v>4</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>160</v>
+        <v>191</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>161</v>
+        <v>192</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="12.75">
@@ -4389,10 +4760,10 @@
         <v>3</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>162</v>
+        <v>193</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>163</v>
+        <v>194</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="12.75">
@@ -4400,10 +4771,10 @@
         <v>2</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>164</v>
+        <v>195</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>165</v>
+        <v>196</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="12.75">
@@ -4411,10 +4782,10 @@
         <v>1</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>166</v>
+        <v>197</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>167</v>
+        <v>198</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="12.75">
@@ -4426,46 +4797,46 @@
     </row>
     <row r="22" spans="1:3" ht="12.75">
       <c r="A22" s="3" t="s">
-        <v>168</v>
+        <v>199</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>169</v>
+        <v>200</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>170</v>
+        <v>201</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="12.75">
       <c r="A23" s="3" t="s">
-        <v>171</v>
+        <v>202</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>153</v>
+        <v>184</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>172</v>
+        <v>203</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="12.75">
       <c r="A24" s="3" t="s">
-        <v>173</v>
+        <v>204</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>151</v>
+        <v>182</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>174</v>
+        <v>205</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="12.75">
       <c r="A25" s="3" t="s">
-        <v>175</v>
+        <v>206</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>149</v>
+        <v>180</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>176</v>
+        <v>207</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="12.75">
@@ -4475,7 +4846,7 @@
     </row>
     <row r="28" spans="1:3" ht="12.75">
       <c r="B28" s="2" t="s">
-        <v>35</v>
+        <v>78</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="12.75">
@@ -4498,15 +4869,15 @@
     </row>
     <row r="33" spans="1:3" ht="12.75">
       <c r="A33" s="2" t="s">
-        <v>177</v>
+        <v>208</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="12.75">
       <c r="B34" s="3" t="s">
-        <v>178</v>
+        <v>209</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>179</v>
+        <v>210</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="12.75">
@@ -4514,23 +4885,23 @@
         <v>19</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>180</v>
+        <v>211</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="12.75">
       <c r="B36" s="3" t="s">
-        <v>181</v>
+        <v>212</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>182</v>
+        <v>213</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="12.75">
       <c r="B37" s="3" t="s">
-        <v>183</v>
+        <v>214</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>184</v>
+        <v>215</v>
       </c>
     </row>
     <row r="40" spans="1:3" ht="12.75">
@@ -4541,36 +4912,36 @@
         <v>14</v>
       </c>
       <c r="C40" t="s">
-        <v>185</v>
+        <v>216</v>
       </c>
     </row>
     <row r="41" spans="1:3" ht="12.75">
       <c r="B41" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="42" spans="1:3" ht="12.75">
       <c r="B42" s="2" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="C42" t="s">
-        <v>186</v>
+        <v>217</v>
       </c>
     </row>
     <row r="43" spans="1:3" ht="12.75">
       <c r="B43" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C43" t="s">
-        <v>187</v>
+        <v>218</v>
       </c>
     </row>
     <row r="45" spans="1:3" ht="15.75" customHeight="1">
       <c r="B45" t="s">
-        <v>188</v>
+        <v>219</v>
       </c>
       <c r="C45" t="s">
-        <v>189</v>
+        <v>220</v>
       </c>
     </row>
   </sheetData>
@@ -4588,18 +4959,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="bed18d5e-33f9-4971-ad53-d046bc7af0c3" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="206edb74-3ff7-4b25-857f-69b348d925d7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <DocumentNotes xmlns="206edb74-3ff7-4b25-857f-69b348d925d7">NewUM project RAID log</DocumentNotes>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100ECD35C65F4987042AD497B5B80201A90" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="eac730192978ca5282e4523680b70cf8">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="206edb74-3ff7-4b25-857f-69b348d925d7" xmlns:ns3="bed18d5e-33f9-4971-ad53-d046bc7af0c3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0a09e63b3e2c946762787fd09a727543" ns2:_="" ns3:_="">
     <xsd:import namespace="206edb74-3ff7-4b25-857f-69b348d925d7"/>
@@ -4802,14 +5161,26 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="bed18d5e-33f9-4971-ad53-d046bc7af0c3" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="206edb74-3ff7-4b25-857f-69b348d925d7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <DocumentNotes xmlns="206edb74-3ff7-4b25-857f-69b348d925d7">NewUM project RAID log</DocumentNotes>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{47DE8F1B-E19C-485B-8A8C-89B734B741BC}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA6E073D-DE16-4674-8469-A47106043DB5}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{48C3B5B6-14EB-4E98-8EBE-710F1EAD96A1}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{48C3B5B6-14EB-4E98-8EBE-710F1EAD96A1}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA6E073D-DE16-4674-8469-A47106043DB5}"/>
 </file>
</xml_diff>